<commit_message>
feat: Enhance backend documentation and API specifications
- Updated backend review fix checklist with atomic role management and audit logging improvements.
- Expanded admin API contract integration to include staff creation and product lifecycle management endpoints.
- Revised sprint execution status to reflect increased functional scope and definition of done metrics.
- Improved admin CRUD coverage documentation to include new user management features and product status transitions.
- Updated database model review document to reflect recent changes in the schema.
- Added new endpoints for archiving and reactivating products and variants in the catalog API.
- Introduced new IAM endpoints for staff user management, including creation, locking, and unlocking functionalities.
- Enhanced OpenAPI specifications to include new schemas and response structures for the updated endpoints.
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -60,6 +60,15 @@
         </r>
       </text>
     </comment>
+    <comment ref="E4" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="H4" authorId="0">
       <text>
         <r>
@@ -69,12 +78,30 @@
         </r>
       </text>
     </comment>
+    <comment ref="I4" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="J4" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DB-20260829-REMOVE-DELETED-AT-V1 · 2026-08-29 · DATABASE+API
 Bỏ deleted_at khỏi 10 model P0 implemented; backfill lifecycle bằng status, thay partial unique index và giữ lịch sử qua audit/FK.
 Sources: migration:20260829233000_remove_deleted_at_v1, document:D22, test:api-unit-and-prisma-validation</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
         </r>
       </text>
     </comment>
@@ -90,9 +117,9 @@
     <comment ref="I5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">DB-20260829-AUTH-ROTATION · 2026-08-29 · DATABASE+API
-Refresh token rotation dùng liên kết rotated_from_id duy nhất; access token được kiểm tra session và permissionVersion từ PostgreSQL.
-Sources: migration:20260829160000_auth_refresh_rotation_guard, OpenAPI:adminLogin/adminRefreshToken/adminLogout/getAdminCurrentUser</t>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
         </r>
       </text>
     </comment>
@@ -141,6 +168,15 @@
         </r>
       </text>
     </comment>
+    <comment ref="E10" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="G10" authorId="0">
       <text>
         <r>
@@ -156,6 +192,15 @@
           <t xml:space="preserve">DB-20260829-AUDIT-HARDENING · 2026-08-29 · DATABASE
 Audit log append-only cho UPDATE/DELETE/TRUNCATE; actor USER bắt buộc có actor_user_id và lịch sử actor dùng FK RESTRICT.
 Sources: migration:20260829170000_audit_log_hardening, test:database-foundation.integration-spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I10" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
         </r>
       </text>
     </comment>
@@ -1416,27 +1461,27 @@
     <comment ref="D7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260829-RBAC-V1 · 2026-08-29 · API+RBAC
-API/UI V1 chỉ expose OWNER GLOBAL và BRANCH_MANAGER/STAFF BRANCH; database giữ WAREHOUSE/OWN dormant cho tương lai. Branch Manager chỉ gán STAFF trong branch được cấp.
-Sources: OpenAPI:listAdminUsers/searchActiveAdminRoles/assignAdminUserRole, document:05-rbac-permissions.csv, test:iam.service.spec.ts</t>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
         </r>
       </text>
     </comment>
     <comment ref="F7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260829-RBAC-V1 · 2026-08-29 · API+RBAC
-API/UI V1 chỉ expose OWNER GLOBAL và BRANCH_MANAGER/STAFF BRANCH; database giữ WAREHOUSE/OWN dormant cho tương lai. Branch Manager chỉ gán STAFF trong branch được cấp.
-Sources: OpenAPI:listAdminUsers/searchActiveAdminRoles/assignAdminUserRole, document:05-rbac-permissions.csv, test:iam.service.spec.ts</t>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
         </r>
       </text>
     </comment>
     <comment ref="G7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260829-RBAC-V1 · 2026-08-29 · API+RBAC
-API/UI V1 chỉ expose OWNER GLOBAL và BRANCH_MANAGER/STAFF BRANCH; database giữ WAREHOUSE/OWN dormant cho tương lai. Branch Manager chỉ gán STAFF trong branch được cấp.
-Sources: OpenAPI:listAdminUsers/searchActiveAdminRoles/assignAdminUserRole, document:05-rbac-permissions.csv, test:iam.service.spec.ts</t>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
         </r>
       </text>
     </comment>
@@ -1933,6 +1978,114 @@
           <t xml:space="preserve">API-20260830-ADMIN-MASTER-CRUD · 2026-08-30 · API+ADMIN+SEED
 Hoàn thiện CRUD lifecycle cho brand/category và branch-one-warehouse: update optimistic version, activate/deactivate có audit; admin dùng generated SDK; bổ sung demo seed idempotent 3 bản ghi mỗi nhóm.
 Sources: OpenAPI:updateAdminBrand/deactivateAdminBrand/activateAdminBrand/updateAdminCategory/deactivateAdminCategory/activateAdminCategory, OpenAPI:updateAdminBranchWithWarehouse/deactivateAdminBranchWithWarehouse/activateAdminBranchWithWarehouse, test:catalog-master.service.spec.ts, test:organization.service.spec.ts, script:prisma/seed-demo.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A10" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260830-STAFF-CATALOG-LIFECYCLE · 2026-08-30 · API+ADMIN+PERSISTENCE-SEMANTICS
+Chốt staff bootstrap bằng email/default password và bổ sung lifecycle archive/reactivate cho Product, Combo qua Product và Variant; Category move chuyển P1.
+Sources: decision:D35/D36/D37, OpenAPI:createAdminStaffUser/archiveAdminProduct/reactivateAdminProduct/archiveAdminProductVariant/reactivateAdminProductVariant, test:iam.service.spec.ts/products.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-creation-drawer.tsx/product-workflow-drawer.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260830-STAFF-CATALOG-LIFECYCLE · 2026-08-30 · API+ADMIN+PERSISTENCE-SEMANTICS
+Chốt staff bootstrap bằng email/default password và bổ sung lifecycle archive/reactivate cho Product, Combo qua Product và Variant; Category move chuyển P1.
+Sources: decision:D35/D36/D37, OpenAPI:createAdminStaffUser/archiveAdminProduct/reactivateAdminProduct/archiveAdminProductVariant/reactivateAdminProductVariant, test:iam.service.spec.ts/products.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-creation-drawer.tsx/product-workflow-drawer.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C10" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260830-STAFF-CATALOG-LIFECYCLE · 2026-08-30 · API+ADMIN+PERSISTENCE-SEMANTICS
+Chốt staff bootstrap bằng email/default password và bổ sung lifecycle archive/reactivate cho Product, Combo qua Product và Variant; Category move chuyển P1.
+Sources: decision:D35/D36/D37, OpenAPI:createAdminStaffUser/archiveAdminProduct/reactivateAdminProduct/archiveAdminProductVariant/reactivateAdminProductVariant, test:iam.service.spec.ts/products.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-creation-drawer.tsx/product-workflow-drawer.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D10" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260830-STAFF-CATALOG-LIFECYCLE · 2026-08-30 · API+ADMIN+PERSISTENCE-SEMANTICS
+Chốt staff bootstrap bằng email/default password và bổ sung lifecycle archive/reactivate cho Product, Combo qua Product và Variant; Category move chuyển P1.
+Sources: decision:D35/D36/D37, OpenAPI:createAdminStaffUser/archiveAdminProduct/reactivateAdminProduct/archiveAdminProductVariant/reactivateAdminProductVariant, test:iam.service.spec.ts/products.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-creation-drawer.tsx/product-workflow-drawer.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E10" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260830-STAFF-CATALOG-LIFECYCLE · 2026-08-30 · API+ADMIN+PERSISTENCE-SEMANTICS
+Chốt staff bootstrap bằng email/default password và bổ sung lifecycle archive/reactivate cho Product, Combo qua Product và Variant; Category move chuyển P1.
+Sources: decision:D35/D36/D37, OpenAPI:createAdminStaffUser/archiveAdminProduct/reactivateAdminProduct/archiveAdminProductVariant/reactivateAdminProductVariant, test:iam.service.spec.ts/products.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-creation-drawer.tsx/product-workflow-drawer.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F10" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260830-STAFF-CATALOG-LIFECYCLE · 2026-08-30 · API+ADMIN+PERSISTENCE-SEMANTICS
+Chốt staff bootstrap bằng email/default password và bổ sung lifecycle archive/reactivate cho Product, Combo qua Product và Variant; Category move chuyển P1.
+Sources: decision:D35/D36/D37, OpenAPI:createAdminStaffUser/archiveAdminProduct/reactivateAdminProduct/archiveAdminProductVariant/reactivateAdminProductVariant, test:iam.service.spec.ts/products.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-creation-drawer.tsx/product-workflow-drawer.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A11" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B11" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C11" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D11" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E11" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F11" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
+Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
+Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
         </r>
       </text>
     </comment>
@@ -2851,7 +3004,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7428" uniqueCount="1427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7440" uniqueCount="1437">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -6537,7 +6690,7 @@
     <t>iam.user.manage</t>
   </si>
   <si>
-    <t>Branch Manager chỉ quản lý STAFF trong branch; không khóa hoặc revoke OWNER cuối cùng</t>
+    <t>OWNER lock/unlock BRANCH_MANAGER và STAFF, không thao tác OWNER; Branch Manager chỉ lock/unlock STAFF trong branch; lock revoke all sessions, unlock reset default password</t>
   </si>
   <si>
     <t>iam.role.view</t>
@@ -7157,6 +7310,42 @@
 test:catalog-master.service.spec.ts
 test:organization.service.spec.ts
 script:prisma/seed-demo.ts</t>
+  </si>
+  <si>
+    <t>API-20260830-STAFF-CATALOG-LIFECYCLE</t>
+  </si>
+  <si>
+    <t>API+ADMIN+PERSISTENCE-SEMANTICS</t>
+  </si>
+  <si>
+    <t>Chốt staff bootstrap bằng email/default password và bổ sung lifecycle archive/reactivate cho Product, Combo qua Product và Variant; Category move chuyển P1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">decision:D35/D36/D37
+OpenAPI:createAdminStaffUser/archiveAdminProduct/reactivateAdminProduct/archiveAdminProductVariant/reactivateAdminProductVariant
+test:iam.service.spec.ts/products.service.spec.ts/admin-contract.e2e-spec.ts
+admin:staff-creation-drawer.tsx/product-workflow-drawer.tsx</t>
+  </si>
+  <si>
+    <t>API-20260901-STAFF-LOCK-UNLOCK</t>
+  </si>
+  <si>
+    <t>2026-09-01</t>
+  </si>
+  <si>
+    <t>API+ADMIN+SECURITY</t>
+  </si>
+  <si>
+    <t>Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenAPI:lockAdminStaffUser/unlockAdminStaffUser
+test:iam.service.spec.ts/admin-contract.e2e-spec.ts
+admin:staff-lifecycle-modal.tsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tables: {"Tên bảng":["users","auth_sessions","audit_logs"]} → Ý nghĩa, Các cột chính
+RBAC Permissions: {"Permission code":"iam.user.manage"} → Allowed scopes, Default roles, Ghi chú</t>
   </si>
 </sst>
 </file>
@@ -7595,7 +7784,7 @@
       <c r="D4" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>64</v>
       </c>
       <c r="F4" s="2" t="s">
@@ -7605,7 +7794,7 @@
       <c r="H4" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="4" t="s">
         <v>66</v>
       </c>
       <c r="J4" s="4" t="s">
@@ -7625,7 +7814,7 @@
       <c r="D5" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F5" s="2" t="s">
@@ -7781,7 +7970,7 @@
       <c r="D10" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="4" t="s">
         <v>101</v>
       </c>
       <c r="F10" s="2" t="s">
@@ -7793,7 +7982,7 @@
       <c r="H10" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="4" t="s">
         <v>104</v>
       </c>
       <c r="J10" s="4" t="s">
@@ -35050,7 +35239,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -35239,6 +35428,46 @@
       </c>
       <c r="F9" s="8" t="s">
         <v>1414</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>1427</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>1423</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>1428</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>1429</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>1430</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>1414</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>1431</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>1432</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>1433</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>1434</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>1435</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>1436</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add revoke role assignment endpoint and update media handling in admin API
- Introduced a new endpoint to revoke role assignments for admin users in the IAM API.
- Added RevokeRoleAssignmentDto schema for request body validation.
- Enhanced media handling in the admin API by adding new properties to MediaAssetDto and ProductMediaDto.
- Updated existing endpoints to include additional response codes for better error handling.
- Extended product detail responses in both admin and storefront APIs to include media and category information.
- Added new DTOs for managing product media and categories.
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -144,27 +144,45 @@
     <comment ref="E9" authorId="0">
       <text>
         <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G9" authorId="0">
+      <text>
+        <r>
           <t xml:space="preserve">API-20260829-RBAC-V1 · 2026-08-29 · API+RBAC
 API/UI V1 chỉ expose OWNER GLOBAL và BRANCH_MANAGER/STAFF BRANCH; database giữ WAREHOUSE/OWN dormant cho tương lai. Branch Manager chỉ gán STAFF trong branch được cấp.
 Sources: OpenAPI:listAdminUsers/searchActiveAdminRoles/assignAdminUserRole, document:05-rbac-permissions.csv, test:iam.service.spec.ts</t>
         </r>
       </text>
     </comment>
-    <comment ref="G9" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">API-20260829-RBAC-V1 · 2026-08-29 · API+RBAC
-API/UI V1 chỉ expose OWNER GLOBAL và BRANCH_MANAGER/STAFF BRANCH; database giữ WAREHOUSE/OWN dormant cho tương lai. Branch Manager chỉ gán STAFF trong branch được cấp.
-Sources: OpenAPI:listAdminUsers/searchActiveAdminRoles/assignAdminUserRole, document:05-rbac-permissions.csv, test:iam.service.spec.ts</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="H9" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260829-RBAC-V1 · 2026-08-29 · API+RBAC
-API/UI V1 chỉ expose OWNER GLOBAL và BRANCH_MANAGER/STAFF BRANCH; database giữ WAREHOUSE/OWN dormant cho tương lai. Branch Manager chỉ gán STAFF trong branch được cấp.
-Sources: OpenAPI:listAdminUsers/searchActiveAdminRoles/assignAdminUserRole, document:05-rbac-permissions.csv, test:iam.service.spec.ts</t>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I9" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J9" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
         </r>
       </text>
     </comment>
@@ -360,13 +378,58 @@
     <comment ref="E18" authorId="0">
       <text>
         <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G18" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DB-20260829-CATALOG-WAVE2 · 2026-08-29 · DATABASE+API
+Catalog Wave 2 được persist: media, brand, category tree, SPU, SKU, product media, global VAT-included price và fixed combo; bổ sung constraint overlap/primary/ownership/no-nesting.
+Sources: migration:20260829180000_catalog_pricing_wave_2, migration:20260829181000_fix_bundle_trigger_functions, OpenAPI:createAdminProduct/createAdminProductVariant/createAdminProductPrice/publishAdminProduct/createAdminProductBundle</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H18" authorId="0">
+      <text>
+        <r>
           <t xml:space="preserve">DBAPI-20260902-PRODUCT-SELLABILITY · 2026-09-02 · DB+API+ADMIN+STOREFRONT
 Tách Product STANDARD/BUNDLE, bundle response theo từng variant, storefront chỉ trả sellable variant và minPrice hợp lệ; publish/combo/variant mutation khóa Product aggregate; giá REGULAR &gt; 0 và có command replace atomic theo expected price id/version.
 Sources: decision:D39/D40/D41, migration:20260902090000_product_sellability_hardening, OpenAPI:searchActiveAdminProductVariants/replaceAdminProductPrice/listCatalogProducts/getCatalogProduct/publishAdminProduct, test:products.service.spec.ts/catalog-schema.integration-spec.ts/admin-contract.e2e-spec.ts</t>
         </r>
       </text>
     </comment>
-    <comment ref="G18" authorId="0">
+    <comment ref="I18" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J18" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E19" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G19" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DB-20260829-CATALOG-WAVE2 · 2026-08-29 · DATABASE+API
@@ -375,7 +438,34 @@
         </r>
       </text>
     </comment>
-    <comment ref="H18" authorId="0">
+    <comment ref="H19" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I19" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J19" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E25" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260902-PRODUCT-SELLABILITY · 2026-09-02 · DB+API+ADMIN+STOREFRONT
@@ -384,7 +474,16 @@
         </r>
       </text>
     </comment>
-    <comment ref="I18" authorId="0">
+    <comment ref="G25" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DB-20260829-CATALOG-WAVE2 · 2026-08-29 · DATABASE+API
+Catalog Wave 2 được persist: media, brand, category tree, SPU, SKU, product media, global VAT-included price và fixed combo; bổ sung constraint overlap/primary/ownership/no-nesting.
+Sources: migration:20260829180000_catalog_pricing_wave_2, migration:20260829181000_fix_bundle_trigger_functions, OpenAPI:createAdminProduct/createAdminProductVariant/createAdminProductPrice/publishAdminProduct/createAdminProductBundle</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H25" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260902-PRODUCT-SELLABILITY · 2026-09-02 · DB+API+ADMIN+STOREFRONT
@@ -393,7 +492,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J18" authorId="0">
+    <comment ref="I25" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260902-PRODUCT-SELLABILITY · 2026-09-02 · DB+API+ADMIN+STOREFRONT
@@ -402,7 +501,25 @@
         </r>
       </text>
     </comment>
-    <comment ref="G19" authorId="0">
+    <comment ref="J25" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260902-PRODUCT-SELLABILITY · 2026-09-02 · DB+API+ADMIN+STOREFRONT
+Tách Product STANDARD/BUNDLE, bundle response theo từng variant, storefront chỉ trả sellable variant và minPrice hợp lệ; publish/combo/variant mutation khóa Product aggregate; giá REGULAR &gt; 0 và có command replace atomic theo expected price id/version.
+Sources: decision:D39/D40/D41, migration:20260902090000_product_sellability_hardening, OpenAPI:searchActiveAdminProductVariants/replaceAdminProductPrice/listCatalogProducts/getCatalogProduct/publishAdminProduct, test:products.service.spec.ts/catalog-schema.integration-spec.ts/admin-contract.e2e-spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E64" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G64" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DB-20260829-CATALOG-WAVE2 · 2026-08-29 · DATABASE+API
@@ -411,111 +528,30 @@
         </r>
       </text>
     </comment>
-    <comment ref="H19" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DB-20260829-REMOVE-DELETED-AT-V1 · 2026-08-29 · DATABASE+API
-Bỏ deleted_at khỏi 10 model P0 implemented; backfill lifecycle bằng status, thay partial unique index và giữ lịch sử qua audit/FK.
-Sources: migration:20260829233000_remove_deleted_at_v1, document:D22, test:api-unit-and-prisma-validation</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I19" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DB-20260829-CATALOG-WAVE2 · 2026-08-29 · DATABASE+API
-Catalog Wave 2 được persist: media, brand, category tree, SPU, SKU, product media, global VAT-included price và fixed combo; bổ sung constraint overlap/primary/ownership/no-nesting.
-Sources: migration:20260829180000_catalog_pricing_wave_2, migration:20260829181000_fix_bundle_trigger_functions, OpenAPI:createAdminProduct/createAdminProductVariant/createAdminProductPrice/publishAdminProduct/createAdminProductBundle</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J19" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DB-20260829-REMOVE-DELETED-AT-V1 · 2026-08-29 · DATABASE+API
-Bỏ deleted_at khỏi 10 model P0 implemented; backfill lifecycle bằng status, thay partial unique index và giữ lịch sử qua audit/FK.
-Sources: migration:20260829233000_remove_deleted_at_v1, document:D22, test:api-unit-and-prisma-validation</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E25" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DBAPI-20260902-PRODUCT-SELLABILITY · 2026-09-02 · DB+API+ADMIN+STOREFRONT
-Tách Product STANDARD/BUNDLE, bundle response theo từng variant, storefront chỉ trả sellable variant và minPrice hợp lệ; publish/combo/variant mutation khóa Product aggregate; giá REGULAR &gt; 0 và có command replace atomic theo expected price id/version.
-Sources: decision:D39/D40/D41, migration:20260902090000_product_sellability_hardening, OpenAPI:searchActiveAdminProductVariants/replaceAdminProductPrice/listCatalogProducts/getCatalogProduct/publishAdminProduct, test:products.service.spec.ts/catalog-schema.integration-spec.ts/admin-contract.e2e-spec.ts</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G25" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DB-20260829-CATALOG-WAVE2 · 2026-08-29 · DATABASE+API
-Catalog Wave 2 được persist: media, brand, category tree, SPU, SKU, product media, global VAT-included price và fixed combo; bổ sung constraint overlap/primary/ownership/no-nesting.
-Sources: migration:20260829180000_catalog_pricing_wave_2, migration:20260829181000_fix_bundle_trigger_functions, OpenAPI:createAdminProduct/createAdminProductVariant/createAdminProductPrice/publishAdminProduct/createAdminProductBundle</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H25" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DBAPI-20260902-PRODUCT-SELLABILITY · 2026-09-02 · DB+API+ADMIN+STOREFRONT
-Tách Product STANDARD/BUNDLE, bundle response theo từng variant, storefront chỉ trả sellable variant và minPrice hợp lệ; publish/combo/variant mutation khóa Product aggregate; giá REGULAR &gt; 0 và có command replace atomic theo expected price id/version.
-Sources: decision:D39/D40/D41, migration:20260902090000_product_sellability_hardening, OpenAPI:searchActiveAdminProductVariants/replaceAdminProductPrice/listCatalogProducts/getCatalogProduct/publishAdminProduct, test:products.service.spec.ts/catalog-schema.integration-spec.ts/admin-contract.e2e-spec.ts</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I25" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DBAPI-20260902-PRODUCT-SELLABILITY · 2026-09-02 · DB+API+ADMIN+STOREFRONT
-Tách Product STANDARD/BUNDLE, bundle response theo từng variant, storefront chỉ trả sellable variant và minPrice hợp lệ; publish/combo/variant mutation khóa Product aggregate; giá REGULAR &gt; 0 và có command replace atomic theo expected price id/version.
-Sources: decision:D39/D40/D41, migration:20260902090000_product_sellability_hardening, OpenAPI:searchActiveAdminProductVariants/replaceAdminProductPrice/listCatalogProducts/getCatalogProduct/publishAdminProduct, test:products.service.spec.ts/catalog-schema.integration-spec.ts/admin-contract.e2e-spec.ts</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J25" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DBAPI-20260902-PRODUCT-SELLABILITY · 2026-09-02 · DB+API+ADMIN+STOREFRONT
-Tách Product STANDARD/BUNDLE, bundle response theo từng variant, storefront chỉ trả sellable variant và minPrice hợp lệ; publish/combo/variant mutation khóa Product aggregate; giá REGULAR &gt; 0 và có command replace atomic theo expected price id/version.
-Sources: decision:D39/D40/D41, migration:20260902090000_product_sellability_hardening, OpenAPI:searchActiveAdminProductVariants/replaceAdminProductPrice/listCatalogProducts/getCatalogProduct/publishAdminProduct, test:products.service.spec.ts/catalog-schema.integration-spec.ts/admin-contract.e2e-spec.ts</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G64" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DB-20260829-CATALOG-WAVE2 · 2026-08-29 · DATABASE+API
-Catalog Wave 2 được persist: media, brand, category tree, SPU, SKU, product media, global VAT-included price và fixed combo; bổ sung constraint overlap/primary/ownership/no-nesting.
-Sources: migration:20260829180000_catalog_pricing_wave_2, migration:20260829181000_fix_bundle_trigger_functions, OpenAPI:createAdminProduct/createAdminProductVariant/createAdminProductPrice/publishAdminProduct/createAdminProductBundle</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="H64" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">DB-20260829-REMOVE-DELETED-AT-V1 · 2026-08-29 · DATABASE+API
-Bỏ deleted_at khỏi 10 model P0 implemented; backfill lifecycle bằng status, thay partial unique index và giữ lịch sử qua audit/FK.
-Sources: migration:20260829233000_remove_deleted_at_v1, document:D22, test:api-unit-and-prisma-validation</t>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
         </r>
       </text>
     </comment>
     <comment ref="I64" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">DB-20260829-CATALOG-WAVE2 · 2026-08-29 · DATABASE+API
-Catalog Wave 2 được persist: media, brand, category tree, SPU, SKU, product media, global VAT-included price và fixed combo; bổ sung constraint overlap/primary/ownership/no-nesting.
-Sources: migration:20260829180000_catalog_pricing_wave_2, migration:20260829181000_fix_bundle_trigger_functions, OpenAPI:createAdminProduct/createAdminProductVariant/createAdminProductPrice/publishAdminProduct/createAdminProductBundle</t>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
         </r>
       </text>
     </comment>
     <comment ref="J64" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">DB-20260829-REMOVE-DELETED-AT-V1 · 2026-08-29 · DATABASE+API
-Bỏ deleted_at khỏi 10 model P0 implemented; backfill lifecycle bằng status, thay partial unique index và giữ lịch sử qua audit/FK.
-Sources: migration:20260829233000_remove_deleted_at_v1, document:D22, test:api-unit-and-prisma-validation</t>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
         </r>
       </text>
     </comment>
@@ -1686,27 +1722,27 @@
     <comment ref="D10" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260829-RBAC-V1 · 2026-08-29 · API+RBAC
-API/UI V1 chỉ expose OWNER GLOBAL và BRANCH_MANAGER/STAFF BRANCH; database giữ WAREHOUSE/OWN dormant cho tương lai. Branch Manager chỉ gán STAFF trong branch được cấp.
-Sources: OpenAPI:listAdminUsers/searchActiveAdminRoles/assignAdminUserRole, document:05-rbac-permissions.csv, test:iam.service.spec.ts</t>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
         </r>
       </text>
     </comment>
     <comment ref="F10" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260829-RBAC-V1 · 2026-08-29 · API+RBAC
-API/UI V1 chỉ expose OWNER GLOBAL và BRANCH_MANAGER/STAFF BRANCH; database giữ WAREHOUSE/OWN dormant cho tương lai. Branch Manager chỉ gán STAFF trong branch được cấp.
-Sources: OpenAPI:listAdminUsers/searchActiveAdminRoles/assignAdminUserRole, document:05-rbac-permissions.csv, test:iam.service.spec.ts</t>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
         </r>
       </text>
     </comment>
     <comment ref="G10" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260829-RBAC-V1 · 2026-08-29 · API+RBAC
-API/UI V1 chỉ expose OWNER GLOBAL và BRANCH_MANAGER/STAFF BRANCH; database giữ WAREHOUSE/OWN dormant cho tương lai. Branch Manager chỉ gán STAFF trong branch được cấp.
-Sources: OpenAPI:listAdminUsers/searchActiveAdminRoles/assignAdminUserRole, document:05-rbac-permissions.csv, test:iam.service.spec.ts</t>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
         </r>
       </text>
     </comment>
@@ -2368,6 +2404,60 @@
         </r>
       </text>
     </comment>
+    <comment ref="A14" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C14" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D14" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E14" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F14" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
+Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
+Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -3283,7 +3373,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7462" uniqueCount="1453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7468" uniqueCount="1458">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -7005,7 +7095,7 @@
     <t>iam.assignment.manage</t>
   </si>
   <si>
-    <t>OWNER gán role hợp lệ; Branch Manager chỉ gán STAFF vào branch được cấp</t>
+    <t>OWNER gán/thu hồi assignment không phải OWNER; Branch Manager chỉ gán/thu hồi STAFF trong branch; thay đổi tăng permissionVersion và audit atomic</t>
   </si>
   <si>
     <t>iam.audit.view</t>
@@ -7686,6 +7776,26 @@
 Tables: {"Tên bảng":"product_prices"} → Ý nghĩa, Unique / CHECK, Các cột chính, Retention
 Columns: {"Tên bảng":"product_prices","Tên cột":"amount"} → Ý nghĩa / trạng thái cho phép
 Columns: upsert {"Tên bảng":"products","Tên cột":"product_type"}</t>
+  </si>
+  <si>
+    <t>API-20260903-SPRINT1-VARIANT-MEDIA-IAM</t>
+  </si>
+  <si>
+    <t>2026-09-03</t>
+  </si>
+  <si>
+    <t>Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment
+test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts
+admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tables: {"Tên bảng":"product_variants"} → Ý nghĩa, Các cột chính, Retention
+Tables: {"Tên bảng":["media_assets","product_media"]} → Ý nghĩa, Unique / CHECK, Các cột chính, Retention
+Tables: {"Tên bảng":"user_role_assignments"} → Ý nghĩa, Unique / CHECK, Các cột chính, Retention
+RBAC Permissions: {"Permission code":"iam.assignment.manage"} → Allowed scopes, Default roles, Ghi chú</t>
   </si>
 </sst>
 </file>
@@ -8290,10 +8400,10 @@
       <c r="H9" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J9" s="4" t="s">
         <v>98</v>
       </c>
     </row>
@@ -8598,7 +8708,7 @@
       <c r="D19" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="4" t="s">
         <v>165</v>
       </c>
       <c r="F19" s="2" t="s">
@@ -10024,7 +10134,7 @@
       <c r="D64" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E64" s="2" t="s">
+      <c r="E64" s="4" t="s">
         <v>455</v>
       </c>
       <c r="F64" s="2" t="s">
@@ -35608,7 +35718,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -35877,6 +35987,26 @@
       </c>
       <c r="F13" s="6" t="s">
         <v>1452</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>1453</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>1454</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>1433</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>1455</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>1456</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>1457</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add break-glass command for bootstrap Admin recovery, update documentation and seed logic
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -63,9 +63,9 @@
     <comment ref="E4" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">DB-20260903-BOOTSTRAP-OWNER · 2026-09-03 · DATABASE+IAM+ADMIN
-Foundation seed tạo đúng một bootstrap OWNER ACTIVE cho local/dev, bắt buộc đổi mật khẩu lần đầu và chỉ khởi tạo password khi record cũ chưa có; rerun seed không ghi đè password đã đổi.
-Sources: seed:api/prisma/seed.ts, decision:D42, admin:login-page.tsx</t>
+          <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
+Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
+Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
@@ -90,13 +90,22 @@
     <comment ref="J4" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">DB-20260903-BOOTSTRAP-OWNER · 2026-09-03 · DATABASE+IAM+ADMIN
-Foundation seed tạo đúng một bootstrap OWNER ACTIVE cho local/dev, bắt buộc đổi mật khẩu lần đầu và chỉ khởi tạo password khi record cũ chưa có; rerun seed không ghi đè password đã đổi.
-Sources: seed:api/prisma/seed.ts, decision:D42, admin:login-page.tsx</t>
+          <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
+Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
+Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
     <comment ref="E5" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
+Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
+Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H5" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260901-CUSTOMER-IDENTITY-V1 · 2026-09-01 · API+STOREFRONT+PERSISTENCE-SEMANTICS
@@ -105,7 +114,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H5" authorId="0">
+    <comment ref="I5" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260901-CUSTOMER-IDENTITY-V1 · 2026-09-01 · API+STOREFRONT+PERSISTENCE-SEMANTICS
@@ -114,12 +123,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="I5" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">API-20260901-CUSTOMER-IDENTITY-V1 · 2026-09-01 · API+STOREFRONT+PERSISTENCE-SEMANTICS
-Public register chỉ tạo CUSTOMER ACTIVE và tạm bỏ verification; yêu cầu email hoặc SĐT; login customer/staff nhận identifier email/phone; email lowercase và SĐT Việt Nam validate metadata đầy đủ rồi lưu E.164. User + GUEST audit + session được tạo atomic.
-Sources: decision:D38, OpenAPI:registerCustomer/loginCustomer/refreshCustomerToken/logoutCustomer/getCustomerCurrentUser/loginAdmin, test:phone-normalization.spec.ts/customer-auth.e2e-spec.ts, client:customer-register-page.tsx/customer-login-page.tsx</t>
+    <comment ref="J5" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
+Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
+Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
@@ -189,22 +198,31 @@
     <comment ref="E10" authorId="0">
       <text>
         <r>
+          <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
+Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
+Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G10" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DB-20260829-AUDIT-HARDENING · 2026-08-29 · DATABASE
+Audit log append-only cho UPDATE/DELETE/TRUNCATE; actor USER bắt buộc có actor_user_id và lịch sử actor dùng FK RESTRICT.
+Sources: migration:20260829170000_audit_log_hardening, test:database-foundation.integration-spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H10" authorId="0">
+      <text>
+        <r>
           <t xml:space="preserve">DBAPI-20260903-AUTH-AUDIT-PRICE-CLOSEOUT · 2026-09-03 · DB+API+ADMIN+STOREFRONT+SECURITY
 Khóa tài khoản atomic ở lần sai mật khẩu thứ 5 và revoke session; staff mới/unlock bắt buộc đổi mật khẩu; refresh token hỗ trợ BODY dev và HttpOnly COOKIE production; audit cursor query GLOBAL owner-only có redaction; price future scheduling/history và rule giảm trên 20% cần reason + OWNER confirm.
 Sources: migration:20260903173000_auth_lockout_and_audit_query, OpenAPI:changeAdminPassword/listAdminAuditLogs/getAdminProductPriceTimeline/createAdminProductPrice/replaceAdminProductPrice, test:auth.service.spec.ts/auth-token-transport.service.spec.ts/audit.service.spec.ts/products.service.spec.ts, admin:change-password-page.tsx/audit-page.tsx/product-price-panel.tsx</t>
         </r>
       </text>
     </comment>
-    <comment ref="G10" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DB-20260829-AUDIT-HARDENING · 2026-08-29 · DATABASE
-Audit log append-only cho UPDATE/DELETE/TRUNCATE; actor USER bắt buộc có actor_user_id và lịch sử actor dùng FK RESTRICT.
-Sources: migration:20260829170000_audit_log_hardening, test:database-foundation.integration-spec.ts</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H10" authorId="0">
+    <comment ref="I10" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260903-AUTH-AUDIT-PRICE-CLOSEOUT · 2026-09-03 · DB+API+ADMIN+STOREFRONT+SECURITY
@@ -213,21 +231,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="I10" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DBAPI-20260903-AUTH-AUDIT-PRICE-CLOSEOUT · 2026-09-03 · DB+API+ADMIN+STOREFRONT+SECURITY
-Khóa tài khoản atomic ở lần sai mật khẩu thứ 5 và revoke session; staff mới/unlock bắt buộc đổi mật khẩu; refresh token hỗ trợ BODY dev và HttpOnly COOKIE production; audit cursor query GLOBAL owner-only có redaction; price future scheduling/history và rule giảm trên 20% cần reason + OWNER confirm.
-Sources: migration:20260903173000_auth_lockout_and_audit_query, OpenAPI:changeAdminPassword/listAdminAuditLogs/getAdminProductPriceTimeline/createAdminProductPrice/replaceAdminProductPrice, test:auth.service.spec.ts/auth-token-transport.service.spec.ts/audit.service.spec.ts/products.service.spec.ts, admin:change-password-page.tsx/audit-page.tsx/product-price-panel.tsx</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="J10" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">DBAPI-20260903-AUTH-AUDIT-PRICE-CLOSEOUT · 2026-09-03 · DB+API+ADMIN+STOREFRONT+SECURITY
-Khóa tài khoản atomic ở lần sai mật khẩu thứ 5 và revoke session; staff mới/unlock bắt buộc đổi mật khẩu; refresh token hỗ trợ BODY dev và HttpOnly COOKIE production; audit cursor query GLOBAL owner-only có redaction; price future scheduling/history và rule giảm trên 20% cần reason + OWNER confirm.
-Sources: migration:20260903173000_auth_lockout_and_audit_query, OpenAPI:changeAdminPassword/listAdminAuditLogs/getAdminProductPriceTimeline/createAdminProductPrice/replaceAdminProductPrice, test:auth.service.spec.ts/auth-token-transport.service.spec.ts/audit.service.spec.ts/products.service.spec.ts, admin:change-password-page.tsx/audit-page.tsx/product-price-panel.tsx</t>
+          <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
+Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
+Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
@@ -3880,6 +3889,60 @@
         </r>
       </text>
     </comment>
+    <comment ref="A19" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
+Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
+Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B19" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
+Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
+Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C19" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
+Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
+Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D19" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
+Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
+Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E19" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
+Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
+Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F19" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
+Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
+Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -4795,7 +4858,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7543" uniqueCount="1500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7549" uniqueCount="1506">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -4989,7 +5052,7 @@
     <t>users</t>
   </si>
   <si>
-    <t>Customer/staff account; local seed có đúng một bootstrap OWNER ACTIVE</t>
+    <t>Customer/staff account; development seed có đúng một bootstrap OWNER; break-glass chỉ phục hồi fixed identity</t>
   </si>
   <si>
     <t>normalized email/phone partial UQ; failed_login_attempts &gt;= 0</t>
@@ -4998,7 +5061,7 @@
     <t>type,email,normalized_email,phone,normalized_phone,password_hash,status,failed_login_attempts,must_change_password,locked_at,lock_reason,permission_version,last_login_at,version</t>
   </si>
   <si>
-    <t>Bootstrap phải đổi password lần đầu; seed không reset password đã đổi; never hard-delete</t>
+    <t>Seed không reset password đã đổi; recovery reset password tạm, bắt đổi password, revoke session và audit; never hard-delete</t>
   </si>
   <si>
     <t>T04</t>
@@ -9368,6 +9431,29 @@
   <si>
     <t xml:space="preserve">Tables: {"Tên bảng":"stock_adjustments"} → Unique / CHECK
 Columns: upsert {"Tên bảng":"stock_adjustments","Tên cột":"adjustment_no"}</t>
+  </si>
+  <si>
+    <t>DBAPI-20260904-BOOTSTRAP-RECOVERY</t>
+  </si>
+  <si>
+    <t>2026-09-04</t>
+  </si>
+  <si>
+    <t>DATABASE+IAM+OPERATIONS</t>
+  </si>
+  <si>
+    <t>Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">command:yarn db:admin:reset
+source:api/src/modules/iam/bootstrap-admin-recovery.ts
+test:bootstrap-admin-recovery.spec.ts
+decision:D42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tables: {"Tên bảng":"users"} → Ý nghĩa, Retention
+Tables: {"Tên bảng":"auth_sessions"} → Ý nghĩa, Retention
+Tables: {"Tên bảng":"audit_logs"} → Ý nghĩa, Retention</t>
   </si>
 </sst>
 </file>
@@ -9851,7 +9937,7 @@
       <c r="I5" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="4" t="s">
         <v>74</v>
       </c>
     </row>
@@ -37455,7 +37541,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -37824,6 +37910,26 @@
       </c>
       <c r="F18" s="6" t="s">
         <v>1499</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>1500</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>1501</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>1502</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>1503</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>1504</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>1505</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: complete Sprint 1 release candidate
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -63,31 +63,67 @@
     <comment ref="E4" authorId="0">
       <text>
         <r>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H4" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260903-AUTH-AUDIT-PRICE-CLOSEOUT · 2026-09-03 · DB+API+ADMIN+STOREFRONT+SECURITY
+Khóa tài khoản atomic ở lần sai mật khẩu thứ 5 và revoke session; staff mới/unlock bắt buộc đổi mật khẩu; refresh token hỗ trợ BODY dev và HttpOnly COOKIE production; audit cursor query GLOBAL owner-only có redaction; price future scheduling/history và rule giảm trên 20% cần reason + OWNER confirm.
+Sources: migration:20260903173000_auth_lockout_and_audit_query, OpenAPI:changeAdminPassword/listAdminAuditLogs/getAdminProductPriceTimeline/createAdminProductPrice/replaceAdminProductPrice, test:auth.service.spec.ts/auth-token-transport.service.spec.ts/audit.service.spec.ts/products.service.spec.ts, admin:change-password-page.tsx/audit-page.tsx/product-price-panel.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I4" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260903-AUTH-AUDIT-PRICE-CLOSEOUT · 2026-09-03 · DB+API+ADMIN+STOREFRONT+SECURITY
+Khóa tài khoản atomic ở lần sai mật khẩu thứ 5 và revoke session; staff mới/unlock bắt buộc đổi mật khẩu; refresh token hỗ trợ BODY dev và HttpOnly COOKIE production; audit cursor query GLOBAL owner-only có redaction; price future scheduling/history và rule giảm trên 20% cần reason + OWNER confirm.
+Sources: migration:20260903173000_auth_lockout_and_audit_query, OpenAPI:changeAdminPassword/listAdminAuditLogs/getAdminProductPriceTimeline/createAdminProductPrice/replaceAdminProductPrice, test:auth.service.spec.ts/auth-token-transport.service.spec.ts/audit.service.spec.ts/products.service.spec.ts, admin:change-password-page.tsx/audit-page.tsx/product-price-panel.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J4" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0">
+      <text>
+        <r>
           <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
 Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
 Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
-    <comment ref="H4" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DBAPI-20260903-AUTH-AUDIT-PRICE-CLOSEOUT · 2026-09-03 · DB+API+ADMIN+STOREFRONT+SECURITY
-Khóa tài khoản atomic ở lần sai mật khẩu thứ 5 và revoke session; staff mới/unlock bắt buộc đổi mật khẩu; refresh token hỗ trợ BODY dev và HttpOnly COOKIE production; audit cursor query GLOBAL owner-only có redaction; price future scheduling/history và rule giảm trên 20% cần reason + OWNER confirm.
-Sources: migration:20260903173000_auth_lockout_and_audit_query, OpenAPI:changeAdminPassword/listAdminAuditLogs/getAdminProductPriceTimeline/createAdminProductPrice/replaceAdminProductPrice, test:auth.service.spec.ts/auth-token-transport.service.spec.ts/audit.service.spec.ts/products.service.spec.ts, admin:change-password-page.tsx/audit-page.tsx/product-price-panel.tsx</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I4" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DBAPI-20260903-AUTH-AUDIT-PRICE-CLOSEOUT · 2026-09-03 · DB+API+ADMIN+STOREFRONT+SECURITY
-Khóa tài khoản atomic ở lần sai mật khẩu thứ 5 và revoke session; staff mới/unlock bắt buộc đổi mật khẩu; refresh token hỗ trợ BODY dev và HttpOnly COOKIE production; audit cursor query GLOBAL owner-only có redaction; price future scheduling/history và rule giảm trên 20% cần reason + OWNER confirm.
-Sources: migration:20260903173000_auth_lockout_and_audit_query, OpenAPI:changeAdminPassword/listAdminAuditLogs/getAdminProductPriceTimeline/createAdminProductPrice/replaceAdminProductPrice, test:auth.service.spec.ts/auth-token-transport.service.spec.ts/audit.service.spec.ts/products.service.spec.ts, admin:change-password-page.tsx/audit-page.tsx/product-price-panel.tsx</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J4" authorId="0">
+    <comment ref="H5" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260901-CUSTOMER-IDENTITY-V1 · 2026-09-01 · API+STOREFRONT+PERSISTENCE-SEMANTICS
+Public register chỉ tạo CUSTOMER ACTIVE và tạm bỏ verification; yêu cầu email hoặc SĐT; login customer/staff nhận identifier email/phone; email lowercase và SĐT Việt Nam validate metadata đầy đủ rồi lưu E.164. User + GUEST audit + session được tạo atomic.
+Sources: decision:D38, OpenAPI:registerCustomer/loginCustomer/refreshCustomerToken/logoutCustomer/getCustomerCurrentUser/loginAdmin, test:phone-normalization.spec.ts/customer-auth.e2e-spec.ts, client:customer-register-page.tsx/customer-login-page.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I5" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260901-CUSTOMER-IDENTITY-V1 · 2026-09-01 · API+STOREFRONT+PERSISTENCE-SEMANTICS
+Public register chỉ tạo CUSTOMER ACTIVE và tạm bỏ verification; yêu cầu email hoặc SĐT; login customer/staff nhận identifier email/phone; email lowercase và SĐT Việt Nam validate metadata đầy đủ rồi lưu E.164. User + GUEST audit + session được tạo atomic.
+Sources: decision:D38, OpenAPI:registerCustomer/loginCustomer/refreshCustomerToken/logoutCustomer/getCustomerCurrentUser/loginAdmin, test:phone-normalization.spec.ts/customer-auth.e2e-spec.ts, client:customer-register-page.tsx/customer-login-page.tsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J5" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
@@ -96,42 +132,6 @@
         </r>
       </text>
     </comment>
-    <comment ref="E5" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
-Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
-Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H5" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">API-20260901-CUSTOMER-IDENTITY-V1 · 2026-09-01 · API+STOREFRONT+PERSISTENCE-SEMANTICS
-Public register chỉ tạo CUSTOMER ACTIVE và tạm bỏ verification; yêu cầu email hoặc SĐT; login customer/staff nhận identifier email/phone; email lowercase và SĐT Việt Nam validate metadata đầy đủ rồi lưu E.164. User + GUEST audit + session được tạo atomic.
-Sources: decision:D38, OpenAPI:registerCustomer/loginCustomer/refreshCustomerToken/logoutCustomer/getCustomerCurrentUser/loginAdmin, test:phone-normalization.spec.ts/customer-auth.e2e-spec.ts, client:customer-register-page.tsx/customer-login-page.tsx</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I5" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">API-20260901-CUSTOMER-IDENTITY-V1 · 2026-09-01 · API+STOREFRONT+PERSISTENCE-SEMANTICS
-Public register chỉ tạo CUSTOMER ACTIVE và tạm bỏ verification; yêu cầu email hoặc SĐT; login customer/staff nhận identifier email/phone; email lowercase và SĐT Việt Nam validate metadata đầy đủ rồi lưu E.164. User + GUEST audit + session được tạo atomic.
-Sources: decision:D38, OpenAPI:registerCustomer/loginCustomer/refreshCustomerToken/logoutCustomer/getCustomerCurrentUser/loginAdmin, test:phone-normalization.spec.ts/customer-auth.e2e-spec.ts, client:customer-register-page.tsx/customer-login-page.tsx</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J5" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">DBAPI-20260904-BOOTSTRAP-RECOVERY · 2026-09-04 · DATABASE+IAM+OPERATIONS
-Bổ sung break-glass command chỉ phục hồi fixed bootstrap OWNER trong development: reset password tạm, ACTIVE, failed attempts, bắt đổi password, tăng permission/version, revoke session và ghi SYSTEM audit trong cùng transaction; foundation seed vẫn không reset credential hiện hữu.
-Sources: command:yarn db:admin:reset, source:api/src/modules/iam/bootstrap-admin-recovery.ts, test:bootstrap-admin-recovery.spec.ts, decision:D42</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="H6" authorId="0">
       <text>
         <r>
@@ -153,22 +153,31 @@
     <comment ref="E9" authorId="0">
       <text>
         <r>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G9" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260829-RBAC-V1 · 2026-08-29 · API+RBAC
+API/UI V1 chỉ expose OWNER GLOBAL và BRANCH_MANAGER/STAFF BRANCH; database giữ WAREHOUSE/OWN dormant cho tương lai. Branch Manager chỉ gán STAFF trong branch được cấp.
+Sources: OpenAPI:listAdminUsers/searchActiveAdminRoles/assignAdminUserRole, document:05-rbac-permissions.csv, test:iam.service.spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H9" authorId="0">
+      <text>
+        <r>
           <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
 Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
 Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
         </r>
       </text>
     </comment>
-    <comment ref="G9" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">API-20260829-RBAC-V1 · 2026-08-29 · API+RBAC
-API/UI V1 chỉ expose OWNER GLOBAL và BRANCH_MANAGER/STAFF BRANCH; database giữ WAREHOUSE/OWN dormant cho tương lai. Branch Manager chỉ gán STAFF trong branch được cấp.
-Sources: OpenAPI:listAdminUsers/searchActiveAdminRoles/assignAdminUserRole, document:05-rbac-permissions.csv, test:iam.service.spec.ts</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H9" authorId="0">
+    <comment ref="I9" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
@@ -177,21 +186,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="I9" authorId="0">
-      <text>
-        <r>
-          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
-Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
-Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="J9" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
-Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
-Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
@@ -2856,81 +2856,81 @@
     <comment ref="D7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
-Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
-Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
     <comment ref="F7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
-Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
-Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
     <comment ref="G7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260901-STAFF-LOCK-UNLOCK · 2026-09-01 · API+ADMIN+SECURITY
-Khóa staff chuyển ACTIVE→LOCKED, tăng permissionVersion và revoke toàn bộ session atomic; mở khóa chuyển LOCKED→ACTIVE, reset Argon2 password về Aa@123456 nhưng không phục hồi session cũ. OWNER không được lock/unlock; Branch Manager chỉ quản lý STAFF trong branch được cấp.
-Sources: OpenAPI:lockAdminStaffUser/unlockAdminStaffUser, test:iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:staff-lifecycle-modal.tsx</t>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
     <comment ref="D8" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260829-RBAC-V1 · 2026-08-29 · API+RBAC
-API/UI V1 chỉ expose OWNER GLOBAL và BRANCH_MANAGER/STAFF BRANCH; database giữ WAREHOUSE/OWN dormant cho tương lai. Branch Manager chỉ gán STAFF trong branch được cấp.
-Sources: OpenAPI:listAdminUsers/searchActiveAdminRoles/assignAdminUserRole, document:05-rbac-permissions.csv, test:iam.service.spec.ts</t>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
     <comment ref="F8" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260829-RBAC-V1 · 2026-08-29 · API+RBAC
-API/UI V1 chỉ expose OWNER GLOBAL và BRANCH_MANAGER/STAFF BRANCH; database giữ WAREHOUSE/OWN dormant cho tương lai. Branch Manager chỉ gán STAFF trong branch được cấp.
-Sources: OpenAPI:listAdminUsers/searchActiveAdminRoles/assignAdminUserRole, document:05-rbac-permissions.csv, test:iam.service.spec.ts</t>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
     <comment ref="G8" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260829-RBAC-V1 · 2026-08-29 · API+RBAC
-API/UI V1 chỉ expose OWNER GLOBAL và BRANCH_MANAGER/STAFF BRANCH; database giữ WAREHOUSE/OWN dormant cho tương lai. Branch Manager chỉ gán STAFF trong branch được cấp.
-Sources: OpenAPI:listAdminUsers/searchActiveAdminRoles/assignAdminUserRole, document:05-rbac-permissions.csv, test:iam.service.spec.ts</t>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
     <comment ref="D10" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
-Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
-Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
     <comment ref="F10" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
-Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
-Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
     <comment ref="G10" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">API-20260903-SPRINT1-VARIANT-MEDIA-IAM · 2026-09-03 · API+ADMIN+PERSISTENCE-SEMANTICS
-Đóng phần quản trị Sprint 1: Product create/update/detail/lifecycle và server pagination; SKU metadata update optimistic với SKU bất biến; Cloudinary finalize persist idempotent và Product Media attach/update/reorder/archive; role assignment revoke giữ history, tăng permissionVersion và audit atomic.
-Sources: OpenAPI:updateAdminProduct/updateAdminProductVariant/finalizeAdminMediaUpload/attachAdminProductMedia/updateAdminProductMedia/reorderAdminProductMedia/archiveAdminProductMedia/revokeAdminUserRoleAssignment, test:media.service.spec.ts/product-media.service.spec.ts/iam.service.spec.ts/admin-contract.e2e-spec.ts, admin:variant-edit-drawer.tsx/product-media-panel.tsx/role-assignment-revoke-modal.tsx</t>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
         </r>
       </text>
     </comment>
@@ -3943,6 +3943,114 @@
         </r>
       </text>
     </comment>
+    <comment ref="A20" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B20" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C20" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D20" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E20" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F20" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBAPI-20260904-SINGLE-ROOT-ADMIN · 2026-09-04 · DATABASE+API+IAM+ADMIN
+Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.
+Sources: OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin, source:api/src/modules/iam/iam.service.ts, source:api/src/modules/auth/auth.service.ts, source:api/src/modules/auth/auth.dto.ts, seed:api/prisma/seed.ts, test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts, decision:D42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A21" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-LOGICAL-DELETE-V1 · 2026-09-05 · API+ADMIN+CATALOG+ORGANIZATION
+Bổ sung sáu HTTP DELETE V1 dưới dạng lifecycle tương thích ngược: branch+warehouse/brand/category chuyển INACTIVE, product/combo chuyển ARCHIVED, variant và product-media chuyển INACTIVE; giữ optimistic version, permission, invariant và audit hiện hữu, không xóa vật lý.
+Sources: OpenAPI:deleteAdminBranchWithWarehouse, OpenAPI:deleteAdminBrand, OpenAPI:deleteAdminCategory, OpenAPI:deleteAdminProduct, OpenAPI:deleteAdminProductVariant, OpenAPI:deleteAdminProductMedia, test:api/src/modules/catalog/logical-delete.controller.spec.ts, decision:D22/D36/D41</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B21" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-LOGICAL-DELETE-V1 · 2026-09-05 · API+ADMIN+CATALOG+ORGANIZATION
+Bổ sung sáu HTTP DELETE V1 dưới dạng lifecycle tương thích ngược: branch+warehouse/brand/category chuyển INACTIVE, product/combo chuyển ARCHIVED, variant và product-media chuyển INACTIVE; giữ optimistic version, permission, invariant và audit hiện hữu, không xóa vật lý.
+Sources: OpenAPI:deleteAdminBranchWithWarehouse, OpenAPI:deleteAdminBrand, OpenAPI:deleteAdminCategory, OpenAPI:deleteAdminProduct, OpenAPI:deleteAdminProductVariant, OpenAPI:deleteAdminProductMedia, test:api/src/modules/catalog/logical-delete.controller.spec.ts, decision:D22/D36/D41</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C21" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-LOGICAL-DELETE-V1 · 2026-09-05 · API+ADMIN+CATALOG+ORGANIZATION
+Bổ sung sáu HTTP DELETE V1 dưới dạng lifecycle tương thích ngược: branch+warehouse/brand/category chuyển INACTIVE, product/combo chuyển ARCHIVED, variant và product-media chuyển INACTIVE; giữ optimistic version, permission, invariant và audit hiện hữu, không xóa vật lý.
+Sources: OpenAPI:deleteAdminBranchWithWarehouse, OpenAPI:deleteAdminBrand, OpenAPI:deleteAdminCategory, OpenAPI:deleteAdminProduct, OpenAPI:deleteAdminProductVariant, OpenAPI:deleteAdminProductMedia, test:api/src/modules/catalog/logical-delete.controller.spec.ts, decision:D22/D36/D41</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D21" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-LOGICAL-DELETE-V1 · 2026-09-05 · API+ADMIN+CATALOG+ORGANIZATION
+Bổ sung sáu HTTP DELETE V1 dưới dạng lifecycle tương thích ngược: branch+warehouse/brand/category chuyển INACTIVE, product/combo chuyển ARCHIVED, variant và product-media chuyển INACTIVE; giữ optimistic version, permission, invariant và audit hiện hữu, không xóa vật lý.
+Sources: OpenAPI:deleteAdminBranchWithWarehouse, OpenAPI:deleteAdminBrand, OpenAPI:deleteAdminCategory, OpenAPI:deleteAdminProduct, OpenAPI:deleteAdminProductVariant, OpenAPI:deleteAdminProductMedia, test:api/src/modules/catalog/logical-delete.controller.spec.ts, decision:D22/D36/D41</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E21" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-LOGICAL-DELETE-V1 · 2026-09-05 · API+ADMIN+CATALOG+ORGANIZATION
+Bổ sung sáu HTTP DELETE V1 dưới dạng lifecycle tương thích ngược: branch+warehouse/brand/category chuyển INACTIVE, product/combo chuyển ARCHIVED, variant và product-media chuyển INACTIVE; giữ optimistic version, permission, invariant và audit hiện hữu, không xóa vật lý.
+Sources: OpenAPI:deleteAdminBranchWithWarehouse, OpenAPI:deleteAdminBrand, OpenAPI:deleteAdminCategory, OpenAPI:deleteAdminProduct, OpenAPI:deleteAdminProductVariant, OpenAPI:deleteAdminProductMedia, test:api/src/modules/catalog/logical-delete.controller.spec.ts, decision:D22/D36/D41</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F21" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-LOGICAL-DELETE-V1 · 2026-09-05 · API+ADMIN+CATALOG+ORGANIZATION
+Bổ sung sáu HTTP DELETE V1 dưới dạng lifecycle tương thích ngược: branch+warehouse/brand/category chuyển INACTIVE, product/combo chuyển ARCHIVED, variant và product-media chuyển INACTIVE; giữ optimistic version, permission, invariant và audit hiện hữu, không xóa vật lý.
+Sources: OpenAPI:deleteAdminBranchWithWarehouse, OpenAPI:deleteAdminBrand, OpenAPI:deleteAdminCategory, OpenAPI:deleteAdminProduct, OpenAPI:deleteAdminProductVariant, OpenAPI:deleteAdminProductMedia, test:api/src/modules/catalog/logical-delete.controller.spec.ts, decision:D22/D36/D41</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -4858,7 +4966,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7549" uniqueCount="1506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7561" uniqueCount="1516">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -5052,7 +5160,7 @@
     <t>users</t>
   </si>
   <si>
-    <t>Customer/staff account; development seed có đúng một bootstrap OWNER; break-glass chỉ phục hồi fixed identity</t>
+    <t>Customer/staff account; development có đúng một fixed bootstrap Admin OWNER</t>
   </si>
   <si>
     <t>normalized email/phone partial UQ; failed_login_attempts &gt;= 0</t>
@@ -5061,7 +5169,7 @@
     <t>type,email,normalized_email,phone,normalized_phone,password_hash,status,failed_login_attempts,must_change_password,locked_at,lock_reason,permission_version,last_login_at,version</t>
   </si>
   <si>
-    <t>Seed không reset password đã đổi; recovery reset password tạm, bắt đổi password, revoke session và audit; never hard-delete</t>
+    <t>OWNER bất biến; Auth trim hai đầu identifier/password; lần sai thứ 5 trả ACCOUNT_LOCKED; login thành công reset attempts; never hard-delete</t>
   </si>
   <si>
     <t>T04</t>
@@ -5142,7 +5250,7 @@
     <t>user_role_assignments</t>
   </si>
   <si>
-    <t>API V1 GLOBAL/BRANCH; DB giữ WAREHOUSE/OWN dormant</t>
+    <t>Một fixed OWNER GLOBAL; BRANCH_MANAGER/STAFF theo BRANCH; WAREHOUSE/OWN dormant</t>
   </si>
   <si>
     <t>user_id-&gt;users; role_id-&gt;roles; branch_id-&gt;branches; warehouse_id-&gt;warehouses</t>
@@ -5154,7 +5262,7 @@
     <t>scope_type,valid_from,valid_to,status,version</t>
   </si>
   <si>
-    <t>audit + expire not delete</t>
+    <t>API cấm gán/thu hồi OWNER; chỉ Admin gốc quản lý assignment cấp dưới; audit + expire not delete</t>
   </si>
   <si>
     <t>T09</t>
@@ -8628,13 +8736,16 @@
     <t>iam.user.manage</t>
   </si>
   <si>
-    <t>OWNER lock/unlock BRANCH_MANAGER và STAFF, không thao tác OWNER; Branch Manager chỉ lock/unlock STAFF trong branch; lock revoke all sessions, unlock reset default password</t>
+    <t>OWNER</t>
+  </si>
+  <si>
+    <t>Chỉ Admin gốc tạo và khóa/mở BRANCH_MANAGER hoặc STAFF; OWNER bất biến</t>
   </si>
   <si>
     <t>iam.role.view</t>
   </si>
   <si>
-    <t>Branch Manager lookup chỉ nhận role STAFF</t>
+    <t>Chỉ Admin gốc lookup BRANCH_MANAGER hoặc STAFF để phân quyền</t>
   </si>
   <si>
     <t>iam.role.manage</t>
@@ -8649,13 +8760,10 @@
     <t>iam.assignment.manage</t>
   </si>
   <si>
-    <t>OWNER gán/thu hồi assignment không phải OWNER; Branch Manager chỉ gán/thu hồi STAFF trong branch; thay đổi tăng permissionVersion và audit atomic</t>
+    <t>Chỉ Admin gốc gán/thu hồi role cấp dưới theo branch; OWNER không thể gán hay thu hồi</t>
   </si>
   <si>
     <t>iam.audit.view</t>
-  </si>
-  <si>
-    <t>OWNER</t>
   </si>
   <si>
     <t>API kiểm tra GLOBAL scope bổ sung; redaction password/token/secret/hash/email/phone; không expose ip/user-agent hash</t>
@@ -9454,6 +9562,53 @@
     <t xml:space="preserve">Tables: {"Tên bảng":"users"} → Ý nghĩa, Retention
 Tables: {"Tên bảng":"auth_sessions"} → Ý nghĩa, Retention
 Tables: {"Tên bảng":"audit_logs"} → Ý nghĩa, Retention</t>
+  </si>
+  <si>
+    <t>DBAPI-20260904-SINGLE-ROOT-ADMIN</t>
+  </si>
+  <si>
+    <t>DATABASE+API+IAM+ADMIN</t>
+  </si>
+  <si>
+    <t>Supersede API-20260829-RBAC-V1: một fixed bootstrap OWNER quản lý account cấp dưới; auto-lock rõ ràng, login reset attempts, Auth trim hai đầu identifier/password và toast Admin không hiện Request ID.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenAPI:createAdminStaffUser/assignAdminUserRole/revokeAdminUserRoleAssignment/loginAdmin
+source:api/src/modules/iam/iam.service.ts
+source:api/src/modules/auth/auth.service.ts
+source:api/src/modules/auth/auth.dto.ts
+seed:api/prisma/seed.ts
+test:iam.service.spec.ts/iam.permissions.spec.ts/auth.service.spec.ts/auth.dto.spec.ts
+decision:D42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tables: {"Tên bảng":"users"} → Ý nghĩa, Retention
+Tables: {"Tên bảng":"user_role_assignments"} → Ý nghĩa, Retention
+RBAC Permissions: {"Permission code":"iam.user.manage"} → Allowed scopes, Default roles, Ghi chú
+RBAC Permissions: {"Permission code":"iam.role.view"} → Allowed scopes, Default roles, Ghi chú
+RBAC Permissions: {"Permission code":"iam.assignment.manage"} → Allowed scopes, Default roles, Ghi chú</t>
+  </si>
+  <si>
+    <t>API-20260905-LOGICAL-DELETE-V1</t>
+  </si>
+  <si>
+    <t>2026-09-05</t>
+  </si>
+  <si>
+    <t>API+ADMIN+CATALOG+ORGANIZATION</t>
+  </si>
+  <si>
+    <t>Bổ sung sáu HTTP DELETE V1 dưới dạng lifecycle tương thích ngược: branch+warehouse/brand/category chuyển INACTIVE, product/combo chuyển ARCHIVED, variant và product-media chuyển INACTIVE; giữ optimistic version, permission, invariant và audit hiện hữu, không xóa vật lý.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenAPI:deleteAdminBranchWithWarehouse
+OpenAPI:deleteAdminBrand
+OpenAPI:deleteAdminCategory
+OpenAPI:deleteAdminProduct
+OpenAPI:deleteAdminProductVariant
+OpenAPI:deleteAdminProductMedia
+test:api/src/modules/catalog/logical-delete.controller.spec.ts
+decision:D22/D36/D41</t>
   </si>
 </sst>
 </file>
@@ -36274,21 +36429,21 @@
         <v>1243</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>1250</v>
+        <v>1239</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>577</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>1253</v>
+        <v>1256</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>1257</v>
+        <v>1258</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>62</v>
@@ -36297,21 +36452,21 @@
         <v>1238</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>1250</v>
+        <v>1239</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>610</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>1253</v>
+        <v>1256</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>1258</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>62</v>
@@ -36326,15 +36481,15 @@
         <v>577</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>1261</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>1262</v>
+        <v>1263</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>62</v>
@@ -36343,21 +36498,21 @@
         <v>1243</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>1250</v>
+        <v>1239</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>577</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>1253</v>
+        <v>1256</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>1264</v>
+        <v>1265</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>62</v>
@@ -36372,7 +36527,7 @@
         <v>577</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>1265</v>
+        <v>1256</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>1266</v>
@@ -37541,7 +37696,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -37930,6 +38085,46 @@
       </c>
       <c r="F19" s="6" t="s">
         <v>1505</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>1506</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>1501</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>1507</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>1508</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>1509</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>1511</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>1513</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>1514</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>1515</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>1441</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: publish admin logical delete contracts
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -4900,13 +4900,67 @@
     <comment ref="A22" authorId="0">
       <text>
         <r>
+          <t xml:space="preserve">API-20260905-ADMIN-DELETE-EXTENSION · 2026-09-05 · API+ADMIN+CMS+REVIEW+IAM
+Bổ sung DELETE logic cho content post (ARCHIVED), review (REJECTED/ẩn) và staff cấp dưới (LOCKED + revoke session/audit); generate OpenAPI/Orval và ghép action xác nhận vào Admin. CMS/Review tiếp tục là in-memory P1, không mô tả sai thành persistence production.
+Sources: OpenAPI:deleteAdminPost, OpenAPI:deleteAdminReview, OpenAPI:deleteAdminStaffUser, test:api/src/modules/cms/cms.service.spec.ts, test:api/src/modules/review/review.service.spec.ts, test:api/src/modules/iam/iam.controller.spec.ts, document:19-admin-api-v1-contract-integration.md, document:21-admin-crud-coverage.md</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B22" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-ADMIN-DELETE-EXTENSION · 2026-09-05 · API+ADMIN+CMS+REVIEW+IAM
+Bổ sung DELETE logic cho content post (ARCHIVED), review (REJECTED/ẩn) và staff cấp dưới (LOCKED + revoke session/audit); generate OpenAPI/Orval và ghép action xác nhận vào Admin. CMS/Review tiếp tục là in-memory P1, không mô tả sai thành persistence production.
+Sources: OpenAPI:deleteAdminPost, OpenAPI:deleteAdminReview, OpenAPI:deleteAdminStaffUser, test:api/src/modules/cms/cms.service.spec.ts, test:api/src/modules/review/review.service.spec.ts, test:api/src/modules/iam/iam.controller.spec.ts, document:19-admin-api-v1-contract-integration.md, document:21-admin-crud-coverage.md</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C22" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-ADMIN-DELETE-EXTENSION · 2026-09-05 · API+ADMIN+CMS+REVIEW+IAM
+Bổ sung DELETE logic cho content post (ARCHIVED), review (REJECTED/ẩn) và staff cấp dưới (LOCKED + revoke session/audit); generate OpenAPI/Orval và ghép action xác nhận vào Admin. CMS/Review tiếp tục là in-memory P1, không mô tả sai thành persistence production.
+Sources: OpenAPI:deleteAdminPost, OpenAPI:deleteAdminReview, OpenAPI:deleteAdminStaffUser, test:api/src/modules/cms/cms.service.spec.ts, test:api/src/modules/review/review.service.spec.ts, test:api/src/modules/iam/iam.controller.spec.ts, document:19-admin-api-v1-contract-integration.md, document:21-admin-crud-coverage.md</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D22" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-ADMIN-DELETE-EXTENSION · 2026-09-05 · API+ADMIN+CMS+REVIEW+IAM
+Bổ sung DELETE logic cho content post (ARCHIVED), review (REJECTED/ẩn) và staff cấp dưới (LOCKED + revoke session/audit); generate OpenAPI/Orval và ghép action xác nhận vào Admin. CMS/Review tiếp tục là in-memory P1, không mô tả sai thành persistence production.
+Sources: OpenAPI:deleteAdminPost, OpenAPI:deleteAdminReview, OpenAPI:deleteAdminStaffUser, test:api/src/modules/cms/cms.service.spec.ts, test:api/src/modules/review/review.service.spec.ts, test:api/src/modules/iam/iam.controller.spec.ts, document:19-admin-api-v1-contract-integration.md, document:21-admin-crud-coverage.md</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E22" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-ADMIN-DELETE-EXTENSION · 2026-09-05 · API+ADMIN+CMS+REVIEW+IAM
+Bổ sung DELETE logic cho content post (ARCHIVED), review (REJECTED/ẩn) và staff cấp dưới (LOCKED + revoke session/audit); generate OpenAPI/Orval và ghép action xác nhận vào Admin. CMS/Review tiếp tục là in-memory P1, không mô tả sai thành persistence production.
+Sources: OpenAPI:deleteAdminPost, OpenAPI:deleteAdminReview, OpenAPI:deleteAdminStaffUser, test:api/src/modules/cms/cms.service.spec.ts, test:api/src/modules/review/review.service.spec.ts, test:api/src/modules/iam/iam.controller.spec.ts, document:19-admin-api-v1-contract-integration.md, document:21-admin-crud-coverage.md</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F22" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-ADMIN-DELETE-EXTENSION · 2026-09-05 · API+ADMIN+CMS+REVIEW+IAM
+Bổ sung DELETE logic cho content post (ARCHIVED), review (REJECTED/ẩn) và staff cấp dưới (LOCKED + revoke session/audit); generate OpenAPI/Orval và ghép action xác nhận vào Admin. CMS/Review tiếp tục là in-memory P1, không mô tả sai thành persistence production.
+Sources: OpenAPI:deleteAdminPost, OpenAPI:deleteAdminReview, OpenAPI:deleteAdminStaffUser, test:api/src/modules/cms/cms.service.spec.ts, test:api/src/modules/review/review.service.spec.ts, test:api/src/modules/iam/iam.controller.spec.ts, document:19-admin-api-v1-contract-integration.md, document:21-admin-crud-coverage.md</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A23" authorId="0">
+      <text>
+        <r>
           <t xml:space="preserve">DBAPI-20260905-BIGINT-IDENTITY · 2026-09-05 · DATABASE+API+ADMIN+STOREFRONT+OPERATIONS
 Supersede D23 bằng D43: entity PK/FK chuyển từ UUIDv7 sang BIGINT IDENTITY do PostgreSQL sinh; API dùng chuỗi số; 21 bảng vật lý giữ UUID cũ ở legacy_id; migration chạy tự động và fail-fast trước khi NestJS listen.
 Sources: decision:D43, migration:20260905120000_migrate_uuid_ids_to_bigint_identity, source:api/src/common/identifiers/entity-id.ts, source:api/scripts/migrate-on-start.cjs, document:23-id-migration-and-startup.md</t>
         </r>
       </text>
     </comment>
-    <comment ref="B22" authorId="0">
+    <comment ref="B23" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260905-BIGINT-IDENTITY · 2026-09-05 · DATABASE+API+ADMIN+STOREFRONT+OPERATIONS
@@ -4915,7 +4969,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C22" authorId="0">
+    <comment ref="C23" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260905-BIGINT-IDENTITY · 2026-09-05 · DATABASE+API+ADMIN+STOREFRONT+OPERATIONS
@@ -4924,7 +4978,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D22" authorId="0">
+    <comment ref="D23" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260905-BIGINT-IDENTITY · 2026-09-05 · DATABASE+API+ADMIN+STOREFRONT+OPERATIONS
@@ -4933,7 +4987,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E22" authorId="0">
+    <comment ref="E23" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260905-BIGINT-IDENTITY · 2026-09-05 · DATABASE+API+ADMIN+STOREFRONT+OPERATIONS
@@ -4942,7 +4996,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F22" authorId="0">
+    <comment ref="F23" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260905-BIGINT-IDENTITY · 2026-09-05 · DATABASE+API+ADMIN+STOREFRONT+OPERATIONS
@@ -5866,7 +5920,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7611" uniqueCount="1525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7617" uniqueCount="1529">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -10521,6 +10575,25 @@
 OpenAPI:deleteAdminProductMedia
 test:api/src/modules/catalog/logical-delete.controller.spec.ts
 decision:D22/D36/D41</t>
+  </si>
+  <si>
+    <t>API-20260905-ADMIN-DELETE-EXTENSION</t>
+  </si>
+  <si>
+    <t>API+ADMIN+CMS+REVIEW+IAM</t>
+  </si>
+  <si>
+    <t>Bổ sung DELETE logic cho content post (ARCHIVED), review (REJECTED/ẩn) và staff cấp dưới (LOCKED + revoke session/audit); generate OpenAPI/Orval và ghép action xác nhận vào Admin. CMS/Review tiếp tục là in-memory P1, không mô tả sai thành persistence production.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenAPI:deleteAdminPost
+OpenAPI:deleteAdminReview
+OpenAPI:deleteAdminStaffUser
+test:api/src/modules/cms/cms.service.spec.ts
+test:api/src/modules/review/review.service.spec.ts
+test:api/src/modules/iam/iam.controller.spec.ts
+document:19-admin-api-v1-contract-integration.md
+document:21-admin-crud-coverage.md</t>
   </si>
   <si>
     <t>DBAPI-20260905-BIGINT-IDENTITY</t>
@@ -38717,7 +38790,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -39165,7 +39238,27 @@
         <v>1523</v>
       </c>
       <c r="F22" s="6" t="s">
+        <v>1445</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
         <v>1524</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>1516</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>1525</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>1526</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>1527</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>1528</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: migrate database during production deploy
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -4900,13 +4900,67 @@
     <comment ref="A22" authorId="0">
       <text>
         <r>
+          <t xml:space="preserve">DBOPS-20260905-VERCEL-AUTO-MIGRATE · 2026-09-05 · DATABASE+DEPLOYMENT+VERCEL
+Production deployment trên Vercel tự chạy prisma migrate deploy trước Nest build; preview/local build không mutate database và có DB_MIGRATE_ON_DEPLOY kill switch.
+Sources: script:api/scripts/migration-execution-policy.cjs, script:api/scripts/migrate-on-start.cjs --deploy, package:@dctd/api#build, test:api/src/database/migration-execution-policy.spec.ts, document:22-repository-split-and-deployment.md@1.4.0, document:23-id-migration-and-startup.md@1.1.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B22" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBOPS-20260905-VERCEL-AUTO-MIGRATE · 2026-09-05 · DATABASE+DEPLOYMENT+VERCEL
+Production deployment trên Vercel tự chạy prisma migrate deploy trước Nest build; preview/local build không mutate database và có DB_MIGRATE_ON_DEPLOY kill switch.
+Sources: script:api/scripts/migration-execution-policy.cjs, script:api/scripts/migrate-on-start.cjs --deploy, package:@dctd/api#build, test:api/src/database/migration-execution-policy.spec.ts, document:22-repository-split-and-deployment.md@1.4.0, document:23-id-migration-and-startup.md@1.1.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C22" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBOPS-20260905-VERCEL-AUTO-MIGRATE · 2026-09-05 · DATABASE+DEPLOYMENT+VERCEL
+Production deployment trên Vercel tự chạy prisma migrate deploy trước Nest build; preview/local build không mutate database và có DB_MIGRATE_ON_DEPLOY kill switch.
+Sources: script:api/scripts/migration-execution-policy.cjs, script:api/scripts/migrate-on-start.cjs --deploy, package:@dctd/api#build, test:api/src/database/migration-execution-policy.spec.ts, document:22-repository-split-and-deployment.md@1.4.0, document:23-id-migration-and-startup.md@1.1.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D22" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBOPS-20260905-VERCEL-AUTO-MIGRATE · 2026-09-05 · DATABASE+DEPLOYMENT+VERCEL
+Production deployment trên Vercel tự chạy prisma migrate deploy trước Nest build; preview/local build không mutate database và có DB_MIGRATE_ON_DEPLOY kill switch.
+Sources: script:api/scripts/migration-execution-policy.cjs, script:api/scripts/migrate-on-start.cjs --deploy, package:@dctd/api#build, test:api/src/database/migration-execution-policy.spec.ts, document:22-repository-split-and-deployment.md@1.4.0, document:23-id-migration-and-startup.md@1.1.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E22" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBOPS-20260905-VERCEL-AUTO-MIGRATE · 2026-09-05 · DATABASE+DEPLOYMENT+VERCEL
+Production deployment trên Vercel tự chạy prisma migrate deploy trước Nest build; preview/local build không mutate database và có DB_MIGRATE_ON_DEPLOY kill switch.
+Sources: script:api/scripts/migration-execution-policy.cjs, script:api/scripts/migrate-on-start.cjs --deploy, package:@dctd/api#build, test:api/src/database/migration-execution-policy.spec.ts, document:22-repository-split-and-deployment.md@1.4.0, document:23-id-migration-and-startup.md@1.1.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F22" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBOPS-20260905-VERCEL-AUTO-MIGRATE · 2026-09-05 · DATABASE+DEPLOYMENT+VERCEL
+Production deployment trên Vercel tự chạy prisma migrate deploy trước Nest build; preview/local build không mutate database và có DB_MIGRATE_ON_DEPLOY kill switch.
+Sources: script:api/scripts/migration-execution-policy.cjs, script:api/scripts/migrate-on-start.cjs --deploy, package:@dctd/api#build, test:api/src/database/migration-execution-policy.spec.ts, document:22-repository-split-and-deployment.md@1.4.0, document:23-id-migration-and-startup.md@1.1.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A23" authorId="0">
+      <text>
+        <r>
           <t xml:space="preserve">API-20260905-ADMIN-DELETE-EXTENSION · 2026-09-05 · API+ADMIN+CMS+REVIEW+IAM
 Bổ sung DELETE logic cho content post (ARCHIVED), review (REJECTED/ẩn) và staff cấp dưới (LOCKED + revoke session/audit); generate OpenAPI/Orval và ghép action xác nhận vào Admin. CMS/Review tiếp tục là in-memory P1, không mô tả sai thành persistence production.
 Sources: OpenAPI:deleteAdminPost, OpenAPI:deleteAdminReview, OpenAPI:deleteAdminStaffUser, test:api/src/modules/cms/cms.service.spec.ts, test:api/src/modules/review/review.service.spec.ts, test:api/src/modules/iam/iam.controller.spec.ts, document:19-admin-api-v1-contract-integration.md, document:21-admin-crud-coverage.md</t>
         </r>
       </text>
     </comment>
-    <comment ref="B22" authorId="0">
+    <comment ref="B23" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260905-ADMIN-DELETE-EXTENSION · 2026-09-05 · API+ADMIN+CMS+REVIEW+IAM
@@ -4915,7 +4969,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C22" authorId="0">
+    <comment ref="C23" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260905-ADMIN-DELETE-EXTENSION · 2026-09-05 · API+ADMIN+CMS+REVIEW+IAM
@@ -4924,7 +4978,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D22" authorId="0">
+    <comment ref="D23" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260905-ADMIN-DELETE-EXTENSION · 2026-09-05 · API+ADMIN+CMS+REVIEW+IAM
@@ -4933,7 +4987,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E22" authorId="0">
+    <comment ref="E23" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260905-ADMIN-DELETE-EXTENSION · 2026-09-05 · API+ADMIN+CMS+REVIEW+IAM
@@ -4942,7 +4996,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F22" authorId="0">
+    <comment ref="F23" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260905-ADMIN-DELETE-EXTENSION · 2026-09-05 · API+ADMIN+CMS+REVIEW+IAM
@@ -4951,7 +5005,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A23" authorId="0">
+    <comment ref="A24" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260905-BIGINT-IDENTITY · 2026-09-05 · DATABASE+API+ADMIN+STOREFRONT+OPERATIONS
@@ -4960,7 +5014,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B23" authorId="0">
+    <comment ref="B24" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260905-BIGINT-IDENTITY · 2026-09-05 · DATABASE+API+ADMIN+STOREFRONT+OPERATIONS
@@ -4969,7 +5023,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C23" authorId="0">
+    <comment ref="C24" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260905-BIGINT-IDENTITY · 2026-09-05 · DATABASE+API+ADMIN+STOREFRONT+OPERATIONS
@@ -4978,7 +5032,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D23" authorId="0">
+    <comment ref="D24" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260905-BIGINT-IDENTITY · 2026-09-05 · DATABASE+API+ADMIN+STOREFRONT+OPERATIONS
@@ -4987,7 +5041,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E23" authorId="0">
+    <comment ref="E24" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260905-BIGINT-IDENTITY · 2026-09-05 · DATABASE+API+ADMIN+STOREFRONT+OPERATIONS
@@ -4996,7 +5050,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F23" authorId="0">
+    <comment ref="F24" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">DBAPI-20260905-BIGINT-IDENTITY · 2026-09-05 · DATABASE+API+ADMIN+STOREFRONT+OPERATIONS
@@ -5920,7 +5974,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7617" uniqueCount="1529">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7623" uniqueCount="1533">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -10575,6 +10629,23 @@
 OpenAPI:deleteAdminProductMedia
 test:api/src/modules/catalog/logical-delete.controller.spec.ts
 decision:D22/D36/D41</t>
+  </si>
+  <si>
+    <t>DBOPS-20260905-VERCEL-AUTO-MIGRATE</t>
+  </si>
+  <si>
+    <t>DATABASE+DEPLOYMENT+VERCEL</t>
+  </si>
+  <si>
+    <t>Production deployment trên Vercel tự chạy prisma migrate deploy trước Nest build; preview/local build không mutate database và có DB_MIGRATE_ON_DEPLOY kill switch.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script:api/scripts/migration-execution-policy.cjs
+script:api/scripts/migrate-on-start.cjs --deploy
+package:@dctd/api#build
+test:api/src/database/migration-execution-policy.spec.ts
+document:22-repository-split-and-deployment.md@1.4.0
+document:23-id-migration-and-startup.md@1.1.0</t>
   </si>
   <si>
     <t>API-20260905-ADMIN-DELETE-EXTENSION</t>
@@ -38790,7 +38861,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -39258,7 +39329,27 @@
         <v>1527</v>
       </c>
       <c r="F23" s="6" t="s">
+        <v>1445</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
         <v>1528</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>1516</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>1529</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>1530</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>1531</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>1532</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add secured Telegram command bot
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -5059,6 +5059,60 @@
         </r>
       </text>
     </comment>
+    <comment ref="A25" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-TELEGRAM-COMMAND-BOT · 2026-09-05 · API+INTEGRATION+OPERATIONS+SECURITY
+Bổ sung Telegram webhook machine-to-machine với secret header, Telegram User ID allowlist và bộ lệnh read-only; endpoint bị loại khỏi OpenAPI dành cho frontend và không cho chạy shell/mutation.
+Sources: route:POST /api/v1/integrations/telegram/webhook, source:api/src/integrations/telegram/telegram-update.service.ts, source:api/src/integrations/telegram/telegram-webhook.controller.ts, test:api/src/integrations/telegram/telegram-update.service.spec.ts, test:api/src/integrations/telegram/telegram-webhook.controller.spec.ts, document:24-telegram-command-bot.md@1.0.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B25" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-TELEGRAM-COMMAND-BOT · 2026-09-05 · API+INTEGRATION+OPERATIONS+SECURITY
+Bổ sung Telegram webhook machine-to-machine với secret header, Telegram User ID allowlist và bộ lệnh read-only; endpoint bị loại khỏi OpenAPI dành cho frontend và không cho chạy shell/mutation.
+Sources: route:POST /api/v1/integrations/telegram/webhook, source:api/src/integrations/telegram/telegram-update.service.ts, source:api/src/integrations/telegram/telegram-webhook.controller.ts, test:api/src/integrations/telegram/telegram-update.service.spec.ts, test:api/src/integrations/telegram/telegram-webhook.controller.spec.ts, document:24-telegram-command-bot.md@1.0.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C25" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-TELEGRAM-COMMAND-BOT · 2026-09-05 · API+INTEGRATION+OPERATIONS+SECURITY
+Bổ sung Telegram webhook machine-to-machine với secret header, Telegram User ID allowlist và bộ lệnh read-only; endpoint bị loại khỏi OpenAPI dành cho frontend và không cho chạy shell/mutation.
+Sources: route:POST /api/v1/integrations/telegram/webhook, source:api/src/integrations/telegram/telegram-update.service.ts, source:api/src/integrations/telegram/telegram-webhook.controller.ts, test:api/src/integrations/telegram/telegram-update.service.spec.ts, test:api/src/integrations/telegram/telegram-webhook.controller.spec.ts, document:24-telegram-command-bot.md@1.0.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D25" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-TELEGRAM-COMMAND-BOT · 2026-09-05 · API+INTEGRATION+OPERATIONS+SECURITY
+Bổ sung Telegram webhook machine-to-machine với secret header, Telegram User ID allowlist và bộ lệnh read-only; endpoint bị loại khỏi OpenAPI dành cho frontend và không cho chạy shell/mutation.
+Sources: route:POST /api/v1/integrations/telegram/webhook, source:api/src/integrations/telegram/telegram-update.service.ts, source:api/src/integrations/telegram/telegram-webhook.controller.ts, test:api/src/integrations/telegram/telegram-update.service.spec.ts, test:api/src/integrations/telegram/telegram-webhook.controller.spec.ts, document:24-telegram-command-bot.md@1.0.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E25" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-TELEGRAM-COMMAND-BOT · 2026-09-05 · API+INTEGRATION+OPERATIONS+SECURITY
+Bổ sung Telegram webhook machine-to-machine với secret header, Telegram User ID allowlist và bộ lệnh read-only; endpoint bị loại khỏi OpenAPI dành cho frontend và không cho chạy shell/mutation.
+Sources: route:POST /api/v1/integrations/telegram/webhook, source:api/src/integrations/telegram/telegram-update.service.ts, source:api/src/integrations/telegram/telegram-webhook.controller.ts, test:api/src/integrations/telegram/telegram-update.service.spec.ts, test:api/src/integrations/telegram/telegram-webhook.controller.spec.ts, document:24-telegram-command-bot.md@1.0.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F25" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-TELEGRAM-COMMAND-BOT · 2026-09-05 · API+INTEGRATION+OPERATIONS+SECURITY
+Bổ sung Telegram webhook machine-to-machine với secret header, Telegram User ID allowlist và bộ lệnh read-only; endpoint bị loại khỏi OpenAPI dành cho frontend và không cho chạy shell/mutation.
+Sources: route:POST /api/v1/integrations/telegram/webhook, source:api/src/integrations/telegram/telegram-update.service.ts, source:api/src/integrations/telegram/telegram-webhook.controller.ts, test:api/src/integrations/telegram/telegram-update.service.spec.ts, test:api/src/integrations/telegram/telegram-webhook.controller.spec.ts, document:24-telegram-command-bot.md@1.0.0</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -5974,7 +6028,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7623" uniqueCount="1533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7629" uniqueCount="1537">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -10686,6 +10740,23 @@
     <t xml:space="preserve">Tables: {"Tên bảng":["branches","warehouses","users","auth_sessions","roles","permissions","user_role_assignments","audit_logs","media_assets","brands","categories","products","product_variants","product_bundles","bundle_items","product_media","product_prices","inventory_balances","inventory_movements","stock_adjustments","stock_adjustment_items"]} → Khóa chính, Khóa ngoại quan trọng
 Columns: {"Tên bảng":["branches","warehouses","users","auth_sessions","roles","permissions","user_role_assignments","audit_logs","media_assets","brands","categories","products","product_variants","product_bundles","bundle_items","product_media","product_prices","inventory_balances","inventory_movements","stock_adjustments","stock_adjustment_items"],"Tên cột":"id"} → Kiểu dữ liệu, Default, Ý nghĩa / trạng thái cho phép
 Columns: {"Tên bảng":["audit_logs","inventory_movements"],"Tên cột":["entity_id","reference_id"]} → Kiểu dữ liệu, Ý nghĩa / trạng thái cho phép</t>
+  </si>
+  <si>
+    <t>API-20260905-TELEGRAM-COMMAND-BOT</t>
+  </si>
+  <si>
+    <t>API+INTEGRATION+OPERATIONS+SECURITY</t>
+  </si>
+  <si>
+    <t>Bổ sung Telegram webhook machine-to-machine với secret header, Telegram User ID allowlist và bộ lệnh read-only; endpoint bị loại khỏi OpenAPI dành cho frontend và không cho chạy shell/mutation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">route:POST /api/v1/integrations/telegram/webhook
+source:api/src/integrations/telegram/telegram-update.service.ts
+source:api/src/integrations/telegram/telegram-webhook.controller.ts
+test:api/src/integrations/telegram/telegram-update.service.spec.ts
+test:api/src/integrations/telegram/telegram-webhook.controller.spec.ts
+document:24-telegram-command-bot.md@1.0.0</t>
   </si>
 </sst>
 </file>
@@ -38861,7 +38932,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -39350,6 +39421,26 @@
       </c>
       <c r="F24" s="6" t="s">
         <v>1532</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
+        <v>1533</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>1516</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>1534</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>1535</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>1536</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>1445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: expose owner permissions in development bypass
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -5113,6 +5113,60 @@
         </r>
       </text>
     </comment>
+    <comment ref="A26" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-DEV-OWNER-PERMISSIONS · 2026-09-05 · API+AUTH+IAM+ADMIN
+Development AUTH_BYPASS principal trả toàn bộ permission OWNER cho cả authentication-only endpoint /admin/auth/me; sửa Admin bị ẩn màn role/phân quyền khi API trả permissions rỗng. Production JWT/RBAC không thay đổi.
+Sources: source:api/src/common/guards/permission.guard.ts#createDevelopmentPrincipal, test:api/src/common/guards/permission.guard.spec.ts, OpenAPI:getAdminCurrentUser, document:19-admin-api-v1-contract-integration.md@1.2.1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B26" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-DEV-OWNER-PERMISSIONS · 2026-09-05 · API+AUTH+IAM+ADMIN
+Development AUTH_BYPASS principal trả toàn bộ permission OWNER cho cả authentication-only endpoint /admin/auth/me; sửa Admin bị ẩn màn role/phân quyền khi API trả permissions rỗng. Production JWT/RBAC không thay đổi.
+Sources: source:api/src/common/guards/permission.guard.ts#createDevelopmentPrincipal, test:api/src/common/guards/permission.guard.spec.ts, OpenAPI:getAdminCurrentUser, document:19-admin-api-v1-contract-integration.md@1.2.1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C26" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-DEV-OWNER-PERMISSIONS · 2026-09-05 · API+AUTH+IAM+ADMIN
+Development AUTH_BYPASS principal trả toàn bộ permission OWNER cho cả authentication-only endpoint /admin/auth/me; sửa Admin bị ẩn màn role/phân quyền khi API trả permissions rỗng. Production JWT/RBAC không thay đổi.
+Sources: source:api/src/common/guards/permission.guard.ts#createDevelopmentPrincipal, test:api/src/common/guards/permission.guard.spec.ts, OpenAPI:getAdminCurrentUser, document:19-admin-api-v1-contract-integration.md@1.2.1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D26" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-DEV-OWNER-PERMISSIONS · 2026-09-05 · API+AUTH+IAM+ADMIN
+Development AUTH_BYPASS principal trả toàn bộ permission OWNER cho cả authentication-only endpoint /admin/auth/me; sửa Admin bị ẩn màn role/phân quyền khi API trả permissions rỗng. Production JWT/RBAC không thay đổi.
+Sources: source:api/src/common/guards/permission.guard.ts#createDevelopmentPrincipal, test:api/src/common/guards/permission.guard.spec.ts, OpenAPI:getAdminCurrentUser, document:19-admin-api-v1-contract-integration.md@1.2.1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E26" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-DEV-OWNER-PERMISSIONS · 2026-09-05 · API+AUTH+IAM+ADMIN
+Development AUTH_BYPASS principal trả toàn bộ permission OWNER cho cả authentication-only endpoint /admin/auth/me; sửa Admin bị ẩn màn role/phân quyền khi API trả permissions rỗng. Production JWT/RBAC không thay đổi.
+Sources: source:api/src/common/guards/permission.guard.ts#createDevelopmentPrincipal, test:api/src/common/guards/permission.guard.spec.ts, OpenAPI:getAdminCurrentUser, document:19-admin-api-v1-contract-integration.md@1.2.1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F26" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260905-DEV-OWNER-PERMISSIONS · 2026-09-05 · API+AUTH+IAM+ADMIN
+Development AUTH_BYPASS principal trả toàn bộ permission OWNER cho cả authentication-only endpoint /admin/auth/me; sửa Admin bị ẩn màn role/phân quyền khi API trả permissions rỗng. Production JWT/RBAC không thay đổi.
+Sources: source:api/src/common/guards/permission.guard.ts#createDevelopmentPrincipal, test:api/src/common/guards/permission.guard.spec.ts, OpenAPI:getAdminCurrentUser, document:19-admin-api-v1-contract-integration.md@1.2.1</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -6028,7 +6082,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7629" uniqueCount="1537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7635" uniqueCount="1541">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -10757,6 +10811,21 @@
 test:api/src/integrations/telegram/telegram-update.service.spec.ts
 test:api/src/integrations/telegram/telegram-webhook.controller.spec.ts
 document:24-telegram-command-bot.md@1.0.0</t>
+  </si>
+  <si>
+    <t>API-20260905-DEV-OWNER-PERMISSIONS</t>
+  </si>
+  <si>
+    <t>API+AUTH+IAM+ADMIN</t>
+  </si>
+  <si>
+    <t>Development AUTH_BYPASS principal trả toàn bộ permission OWNER cho cả authentication-only endpoint /admin/auth/me; sửa Admin bị ẩn màn role/phân quyền khi API trả permissions rỗng. Production JWT/RBAC không thay đổi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">source:api/src/common/guards/permission.guard.ts#createDevelopmentPrincipal
+test:api/src/common/guards/permission.guard.spec.ts
+OpenAPI:getAdminCurrentUser
+document:19-admin-api-v1-contract-integration.md@1.2.1</t>
   </si>
 </sst>
 </file>
@@ -38932,7 +39001,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -39440,6 +39509,26 @@
         <v>1536</v>
       </c>
       <c r="F25" s="6" t="s">
+        <v>1445</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
+        <v>1537</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>1516</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>1538</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>1539</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>1540</v>
+      </c>
+      <c r="F26" s="6" t="s">
         <v>1445</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: control Codex tasks through Telegram
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -5167,6 +5167,60 @@
         </r>
       </text>
     </comment>
+    <comment ref="A27" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">OPS-20260905-TELEGRAM-CODEX-WORKER · 2026-09-05 · OPERATIONS+SECURITY+DEVELOPER-TOOLING
+Bổ sung local polling worker cho phép OWNER tạo và xác nhận task Codex qua Telegram trên ba repository cố định; dùng workspace-write sandbox, loại secret env, lưu state local và gửi notification chủ động. Không thay đổi database hoặc public API/OpenAPI.
+Sources: source:api/scripts/telegram-codex-worker.ts, source:api/scripts/telegram-notify.ts, source:api/src/integrations/telegram/codex-bridge, test:api/src/integrations/telegram/codex-bridge/codex-command.parser.spec.ts, test:api/src/integrations/telegram/codex-bridge/codex-process.runner.spec.ts, test:api/src/integrations/telegram/codex-bridge/codex-task.store.spec.ts, document:24-telegram-command-bot.md@1.1.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B27" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">OPS-20260905-TELEGRAM-CODEX-WORKER · 2026-09-05 · OPERATIONS+SECURITY+DEVELOPER-TOOLING
+Bổ sung local polling worker cho phép OWNER tạo và xác nhận task Codex qua Telegram trên ba repository cố định; dùng workspace-write sandbox, loại secret env, lưu state local và gửi notification chủ động. Không thay đổi database hoặc public API/OpenAPI.
+Sources: source:api/scripts/telegram-codex-worker.ts, source:api/scripts/telegram-notify.ts, source:api/src/integrations/telegram/codex-bridge, test:api/src/integrations/telegram/codex-bridge/codex-command.parser.spec.ts, test:api/src/integrations/telegram/codex-bridge/codex-process.runner.spec.ts, test:api/src/integrations/telegram/codex-bridge/codex-task.store.spec.ts, document:24-telegram-command-bot.md@1.1.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C27" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">OPS-20260905-TELEGRAM-CODEX-WORKER · 2026-09-05 · OPERATIONS+SECURITY+DEVELOPER-TOOLING
+Bổ sung local polling worker cho phép OWNER tạo và xác nhận task Codex qua Telegram trên ba repository cố định; dùng workspace-write sandbox, loại secret env, lưu state local và gửi notification chủ động. Không thay đổi database hoặc public API/OpenAPI.
+Sources: source:api/scripts/telegram-codex-worker.ts, source:api/scripts/telegram-notify.ts, source:api/src/integrations/telegram/codex-bridge, test:api/src/integrations/telegram/codex-bridge/codex-command.parser.spec.ts, test:api/src/integrations/telegram/codex-bridge/codex-process.runner.spec.ts, test:api/src/integrations/telegram/codex-bridge/codex-task.store.spec.ts, document:24-telegram-command-bot.md@1.1.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D27" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">OPS-20260905-TELEGRAM-CODEX-WORKER · 2026-09-05 · OPERATIONS+SECURITY+DEVELOPER-TOOLING
+Bổ sung local polling worker cho phép OWNER tạo và xác nhận task Codex qua Telegram trên ba repository cố định; dùng workspace-write sandbox, loại secret env, lưu state local và gửi notification chủ động. Không thay đổi database hoặc public API/OpenAPI.
+Sources: source:api/scripts/telegram-codex-worker.ts, source:api/scripts/telegram-notify.ts, source:api/src/integrations/telegram/codex-bridge, test:api/src/integrations/telegram/codex-bridge/codex-command.parser.spec.ts, test:api/src/integrations/telegram/codex-bridge/codex-process.runner.spec.ts, test:api/src/integrations/telegram/codex-bridge/codex-task.store.spec.ts, document:24-telegram-command-bot.md@1.1.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E27" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">OPS-20260905-TELEGRAM-CODEX-WORKER · 2026-09-05 · OPERATIONS+SECURITY+DEVELOPER-TOOLING
+Bổ sung local polling worker cho phép OWNER tạo và xác nhận task Codex qua Telegram trên ba repository cố định; dùng workspace-write sandbox, loại secret env, lưu state local và gửi notification chủ động. Không thay đổi database hoặc public API/OpenAPI.
+Sources: source:api/scripts/telegram-codex-worker.ts, source:api/scripts/telegram-notify.ts, source:api/src/integrations/telegram/codex-bridge, test:api/src/integrations/telegram/codex-bridge/codex-command.parser.spec.ts, test:api/src/integrations/telegram/codex-bridge/codex-process.runner.spec.ts, test:api/src/integrations/telegram/codex-bridge/codex-task.store.spec.ts, document:24-telegram-command-bot.md@1.1.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F27" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">OPS-20260905-TELEGRAM-CODEX-WORKER · 2026-09-05 · OPERATIONS+SECURITY+DEVELOPER-TOOLING
+Bổ sung local polling worker cho phép OWNER tạo và xác nhận task Codex qua Telegram trên ba repository cố định; dùng workspace-write sandbox, loại secret env, lưu state local và gửi notification chủ động. Không thay đổi database hoặc public API/OpenAPI.
+Sources: source:api/scripts/telegram-codex-worker.ts, source:api/scripts/telegram-notify.ts, source:api/src/integrations/telegram/codex-bridge, test:api/src/integrations/telegram/codex-bridge/codex-command.parser.spec.ts, test:api/src/integrations/telegram/codex-bridge/codex-process.runner.spec.ts, test:api/src/integrations/telegram/codex-bridge/codex-task.store.spec.ts, document:24-telegram-command-bot.md@1.1.0</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -6082,7 +6136,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7635" uniqueCount="1541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7641" uniqueCount="1545">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -10826,6 +10880,24 @@
 test:api/src/common/guards/permission.guard.spec.ts
 OpenAPI:getAdminCurrentUser
 document:19-admin-api-v1-contract-integration.md@1.2.1</t>
+  </si>
+  <si>
+    <t>OPS-20260905-TELEGRAM-CODEX-WORKER</t>
+  </si>
+  <si>
+    <t>OPERATIONS+SECURITY+DEVELOPER-TOOLING</t>
+  </si>
+  <si>
+    <t>Bổ sung local polling worker cho phép OWNER tạo và xác nhận task Codex qua Telegram trên ba repository cố định; dùng workspace-write sandbox, loại secret env, lưu state local và gửi notification chủ động. Không thay đổi database hoặc public API/OpenAPI.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">source:api/scripts/telegram-codex-worker.ts
+source:api/scripts/telegram-notify.ts
+source:api/src/integrations/telegram/codex-bridge
+test:api/src/integrations/telegram/codex-bridge/codex-command.parser.spec.ts
+test:api/src/integrations/telegram/codex-bridge/codex-process.runner.spec.ts
+test:api/src/integrations/telegram/codex-bridge/codex-task.store.spec.ts
+document:24-telegram-command-bot.md@1.1.0</t>
   </si>
 </sst>
 </file>
@@ -39001,7 +39073,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -39529,6 +39601,26 @@
         <v>1540</v>
       </c>
       <c r="F26" s="6" t="s">
+        <v>1445</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>1541</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>1516</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>1542</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>1543</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>1544</v>
+      </c>
+      <c r="F27" s="6" t="s">
         <v>1445</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(config): default authorization bypass to disabled
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -7084,6 +7084,60 @@
         </r>
       </text>
     </comment>
+    <comment ref="A35" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260906-AUTH-BYPASS-DENY-DEFAULT · 2026-09-06 · API+SECURITY-CONFIG+DEPLOYMENT
+AUTH_BYPASS mặc định false trong validation và application config; development phải opt-in tường minh, production không còn crash khi Vercel không khai báo biến tùy chọn này.
+Sources: source:src/config/env.validation.ts, source:src/config/app.config.ts, test:src/config/env.validation.spec.ts, document:22-repository-split-and-deployment.md@1.4.1, evidence:Vercel FUNCTION_INVOCATION_FAILED 2026-09-06T09:29:57Z</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B35" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260906-AUTH-BYPASS-DENY-DEFAULT · 2026-09-06 · API+SECURITY-CONFIG+DEPLOYMENT
+AUTH_BYPASS mặc định false trong validation và application config; development phải opt-in tường minh, production không còn crash khi Vercel không khai báo biến tùy chọn này.
+Sources: source:src/config/env.validation.ts, source:src/config/app.config.ts, test:src/config/env.validation.spec.ts, document:22-repository-split-and-deployment.md@1.4.1, evidence:Vercel FUNCTION_INVOCATION_FAILED 2026-09-06T09:29:57Z</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C35" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260906-AUTH-BYPASS-DENY-DEFAULT · 2026-09-06 · API+SECURITY-CONFIG+DEPLOYMENT
+AUTH_BYPASS mặc định false trong validation và application config; development phải opt-in tường minh, production không còn crash khi Vercel không khai báo biến tùy chọn này.
+Sources: source:src/config/env.validation.ts, source:src/config/app.config.ts, test:src/config/env.validation.spec.ts, document:22-repository-split-and-deployment.md@1.4.1, evidence:Vercel FUNCTION_INVOCATION_FAILED 2026-09-06T09:29:57Z</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D35" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260906-AUTH-BYPASS-DENY-DEFAULT · 2026-09-06 · API+SECURITY-CONFIG+DEPLOYMENT
+AUTH_BYPASS mặc định false trong validation và application config; development phải opt-in tường minh, production không còn crash khi Vercel không khai báo biến tùy chọn này.
+Sources: source:src/config/env.validation.ts, source:src/config/app.config.ts, test:src/config/env.validation.spec.ts, document:22-repository-split-and-deployment.md@1.4.1, evidence:Vercel FUNCTION_INVOCATION_FAILED 2026-09-06T09:29:57Z</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E35" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260906-AUTH-BYPASS-DENY-DEFAULT · 2026-09-06 · API+SECURITY-CONFIG+DEPLOYMENT
+AUTH_BYPASS mặc định false trong validation và application config; development phải opt-in tường minh, production không còn crash khi Vercel không khai báo biến tùy chọn này.
+Sources: source:src/config/env.validation.ts, source:src/config/app.config.ts, test:src/config/env.validation.spec.ts, document:22-repository-split-and-deployment.md@1.4.1, evidence:Vercel FUNCTION_INVOCATION_FAILED 2026-09-06T09:29:57Z</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F35" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260906-AUTH-BYPASS-DENY-DEFAULT · 2026-09-06 · API+SECURITY-CONFIG+DEPLOYMENT
+AUTH_BYPASS mặc định false trong validation và application config; development phải opt-in tường minh, production không còn crash khi Vercel không khai báo biến tùy chọn này.
+Sources: source:src/config/env.validation.ts, source:src/config/app.config.ts, test:src/config/env.validation.spec.ts, document:22-repository-split-and-deployment.md@1.4.1, evidence:Vercel FUNCTION_INVOCATION_FAILED 2026-09-06T09:29:57Z</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -7999,7 +8053,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7756" uniqueCount="1603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7762" uniqueCount="1607">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -12982,6 +13036,22 @@
 RBAC Permissions: upsert {"Permission code":"inventory.transfer.create"}
 RBAC Permissions: upsert {"Permission code":"inventory.transfer.ship"}
 RBAC Permissions: upsert {"Permission code":"inventory.transfer.receive"}</t>
+  </si>
+  <si>
+    <t>API-20260906-AUTH-BYPASS-DENY-DEFAULT</t>
+  </si>
+  <si>
+    <t>API+SECURITY-CONFIG+DEPLOYMENT</t>
+  </si>
+  <si>
+    <t>AUTH_BYPASS mặc định false trong validation và application config; development phải opt-in tường minh, production không còn crash khi Vercel không khai báo biến tùy chọn này.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">source:src/config/env.validation.ts
+source:src/config/app.config.ts
+test:src/config/env.validation.spec.ts
+document:22-repository-split-and-deployment.md@1.4.1
+evidence:Vercel FUNCTION_INVOCATION_FAILED 2026-09-06T09:29:57Z</t>
   </si>
 </sst>
 </file>
@@ -41330,7 +41400,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -42019,6 +42089,26 @@
       </c>
       <c r="F34" s="6" t="s">
         <v>1602</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>1603</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>1588</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>1604</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>1605</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>1606</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>1468</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(auth): allow authenticated me endpoint
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -7138,6 +7138,60 @@
         </r>
       </text>
     </comment>
+    <comment ref="A36" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260906-AUTH-ME-GUARD-FIX · 2026-09-06 · API+SECURITY+DEPLOYMENT+TEST
+Sửa PermissionGuard production gọi every trên permission metadata undefined tại endpoint authentication-only, khiến /admin/auth/me trả 500 sau login; thêm regression test, internal 5xx logging theo request ID và redact Vercel authentication headers.
+Sources: source:src/common/guards/permission.guard.ts, source:src/common/filters/http-exception.filter.ts, source:src/app.module.ts, test:src/common/guards/permission.guard.spec.ts, document:19-admin-api-v1-contract-integration.md@1.2.2, document:22-repository-split-and-deployment.md@1.4.2, evidence:local login 200 then auth/me 200 against shared Supabase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B36" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260906-AUTH-ME-GUARD-FIX · 2026-09-06 · API+SECURITY+DEPLOYMENT+TEST
+Sửa PermissionGuard production gọi every trên permission metadata undefined tại endpoint authentication-only, khiến /admin/auth/me trả 500 sau login; thêm regression test, internal 5xx logging theo request ID và redact Vercel authentication headers.
+Sources: source:src/common/guards/permission.guard.ts, source:src/common/filters/http-exception.filter.ts, source:src/app.module.ts, test:src/common/guards/permission.guard.spec.ts, document:19-admin-api-v1-contract-integration.md@1.2.2, document:22-repository-split-and-deployment.md@1.4.2, evidence:local login 200 then auth/me 200 against shared Supabase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C36" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260906-AUTH-ME-GUARD-FIX · 2026-09-06 · API+SECURITY+DEPLOYMENT+TEST
+Sửa PermissionGuard production gọi every trên permission metadata undefined tại endpoint authentication-only, khiến /admin/auth/me trả 500 sau login; thêm regression test, internal 5xx logging theo request ID và redact Vercel authentication headers.
+Sources: source:src/common/guards/permission.guard.ts, source:src/common/filters/http-exception.filter.ts, source:src/app.module.ts, test:src/common/guards/permission.guard.spec.ts, document:19-admin-api-v1-contract-integration.md@1.2.2, document:22-repository-split-and-deployment.md@1.4.2, evidence:local login 200 then auth/me 200 against shared Supabase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D36" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260906-AUTH-ME-GUARD-FIX · 2026-09-06 · API+SECURITY+DEPLOYMENT+TEST
+Sửa PermissionGuard production gọi every trên permission metadata undefined tại endpoint authentication-only, khiến /admin/auth/me trả 500 sau login; thêm regression test, internal 5xx logging theo request ID và redact Vercel authentication headers.
+Sources: source:src/common/guards/permission.guard.ts, source:src/common/filters/http-exception.filter.ts, source:src/app.module.ts, test:src/common/guards/permission.guard.spec.ts, document:19-admin-api-v1-contract-integration.md@1.2.2, document:22-repository-split-and-deployment.md@1.4.2, evidence:local login 200 then auth/me 200 against shared Supabase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E36" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260906-AUTH-ME-GUARD-FIX · 2026-09-06 · API+SECURITY+DEPLOYMENT+TEST
+Sửa PermissionGuard production gọi every trên permission metadata undefined tại endpoint authentication-only, khiến /admin/auth/me trả 500 sau login; thêm regression test, internal 5xx logging theo request ID và redact Vercel authentication headers.
+Sources: source:src/common/guards/permission.guard.ts, source:src/common/filters/http-exception.filter.ts, source:src/app.module.ts, test:src/common/guards/permission.guard.spec.ts, document:19-admin-api-v1-contract-integration.md@1.2.2, document:22-repository-split-and-deployment.md@1.4.2, evidence:local login 200 then auth/me 200 against shared Supabase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F36" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260906-AUTH-ME-GUARD-FIX · 2026-09-06 · API+SECURITY+DEPLOYMENT+TEST
+Sửa PermissionGuard production gọi every trên permission metadata undefined tại endpoint authentication-only, khiến /admin/auth/me trả 500 sau login; thêm regression test, internal 5xx logging theo request ID và redact Vercel authentication headers.
+Sources: source:src/common/guards/permission.guard.ts, source:src/common/filters/http-exception.filter.ts, source:src/app.module.ts, test:src/common/guards/permission.guard.spec.ts, document:19-admin-api-v1-contract-integration.md@1.2.2, document:22-repository-split-and-deployment.md@1.4.2, evidence:local login 200 then auth/me 200 against shared Supabase</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -8053,7 +8107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7762" uniqueCount="1607">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7768" uniqueCount="1611">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -13052,6 +13106,24 @@
 test:src/config/env.validation.spec.ts
 document:22-repository-split-and-deployment.md@1.4.1
 evidence:Vercel FUNCTION_INVOCATION_FAILED 2026-09-06T09:29:57Z</t>
+  </si>
+  <si>
+    <t>API-20260906-AUTH-ME-GUARD-FIX</t>
+  </si>
+  <si>
+    <t>API+SECURITY+DEPLOYMENT+TEST</t>
+  </si>
+  <si>
+    <t>Sửa PermissionGuard production gọi every trên permission metadata undefined tại endpoint authentication-only, khiến /admin/auth/me trả 500 sau login; thêm regression test, internal 5xx logging theo request ID và redact Vercel authentication headers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">source:src/common/guards/permission.guard.ts
+source:src/common/filters/http-exception.filter.ts
+source:src/app.module.ts
+test:src/common/guards/permission.guard.spec.ts
+document:19-admin-api-v1-contract-integration.md@1.2.2
+document:22-repository-split-and-deployment.md@1.4.2
+evidence:local login 200 then auth/me 200 against shared Supabase</t>
   </si>
 </sst>
 </file>
@@ -41400,7 +41472,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -42108,6 +42180,26 @@
         <v>1606</v>
       </c>
       <c r="F35" s="6" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
+        <v>1607</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>1588</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>1608</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>1609</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>1610</v>
+      </c>
+      <c r="F36" s="6" t="s">
         <v>1468</v>
       </c>
     </row>

</xml_diff>

<commit_message>
test(inventory): cover ledger cursor pagination
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -4899,6 +4899,52 @@
 </comments>
 </file>
 
+<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="C12" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">D11-SYNC-20260907 · 2026-09-07 · DECISION+DOCUMENTATION
+Đồng bộ D11 từ PROPOSED sang DECIDED theo rule Sprint 2 đã chốt và triển khai: V1 không maker-checker; BRANCH_MANAGER giảm tối đa 10 đơn vị/SKU/lệnh; GLOBAL/OWNER được vượt; reason và audit luôn bắt buộc.
+Sources: decision:D11, document:08-open-decisions.csv, document:25-sprint-2-execution-status.md@1.2.1, source:src/modules/inventory/inventory.service.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D12" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">D11-SYNC-20260907 · 2026-09-07 · DECISION+DOCUMENTATION
+Đồng bộ D11 từ PROPOSED sang DECIDED theo rule Sprint 2 đã chốt và triển khai: V1 không maker-checker; BRANCH_MANAGER giảm tối đa 10 đơn vị/SKU/lệnh; GLOBAL/OWNER được vượt; reason và audit luôn bắt buộc.
+Sources: decision:D11, document:08-open-decisions.csv, document:25-sprint-2-execution-status.md@1.2.1, source:src/modules/inventory/inventory.service.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G12" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">D11-SYNC-20260907 · 2026-09-07 · DECISION+DOCUMENTATION
+Đồng bộ D11 từ PROPOSED sang DECIDED theo rule Sprint 2 đã chốt và triển khai: V1 không maker-checker; BRANCH_MANAGER giảm tối đa 10 đơn vị/SKU/lệnh; GLOBAL/OWNER được vượt; reason và audit luôn bắt buộc.
+Sources: decision:D11, document:08-open-decisions.csv, document:25-sprint-2-execution-status.md@1.2.1, source:src/modules/inventory/inventory.service.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H12" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">D11-SYNC-20260907 · 2026-09-07 · DECISION+DOCUMENTATION
+Đồng bộ D11 từ PROPOSED sang DECIDED theo rule Sprint 2 đã chốt và triển khai: V1 không maker-checker; BRANCH_MANAGER giảm tối đa 10 đơn vị/SKU/lệnh; GLOBAL/OWNER được vượt; reason và audit luôn bắt buộc.
+Sources: decision:D11, document:08-open-decisions.csv, document:25-sprint-2-execution-status.md@1.2.1, source:src/modules/inventory/inventory.service.ts</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
@@ -7192,6 +7238,114 @@
         </r>
       </text>
     </comment>
+    <comment ref="A37" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">S2-LEDGER-CURSOR-HTTP-20260907 · 2026-09-07 · API-TEST+DOCUMENTATION
+Bổ sung HTTP E2E regression cho inventory movement cursor: trang đầu trả opaque nextCursor, trang kế tiếp không lặp record và malformed cursor vẫn trả 400; không đổi schema hoặc API contract.
+Sources: test:test/admin-contract.e2e-spec.ts, operation:listInventoryMovements, document:25-sprint-2-execution-status.md@1.2.1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B37" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">S2-LEDGER-CURSOR-HTTP-20260907 · 2026-09-07 · API-TEST+DOCUMENTATION
+Bổ sung HTTP E2E regression cho inventory movement cursor: trang đầu trả opaque nextCursor, trang kế tiếp không lặp record và malformed cursor vẫn trả 400; không đổi schema hoặc API contract.
+Sources: test:test/admin-contract.e2e-spec.ts, operation:listInventoryMovements, document:25-sprint-2-execution-status.md@1.2.1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C37" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">S2-LEDGER-CURSOR-HTTP-20260907 · 2026-09-07 · API-TEST+DOCUMENTATION
+Bổ sung HTTP E2E regression cho inventory movement cursor: trang đầu trả opaque nextCursor, trang kế tiếp không lặp record và malformed cursor vẫn trả 400; không đổi schema hoặc API contract.
+Sources: test:test/admin-contract.e2e-spec.ts, operation:listInventoryMovements, document:25-sprint-2-execution-status.md@1.2.1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D37" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">S2-LEDGER-CURSOR-HTTP-20260907 · 2026-09-07 · API-TEST+DOCUMENTATION
+Bổ sung HTTP E2E regression cho inventory movement cursor: trang đầu trả opaque nextCursor, trang kế tiếp không lặp record và malformed cursor vẫn trả 400; không đổi schema hoặc API contract.
+Sources: test:test/admin-contract.e2e-spec.ts, operation:listInventoryMovements, document:25-sprint-2-execution-status.md@1.2.1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E37" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">S2-LEDGER-CURSOR-HTTP-20260907 · 2026-09-07 · API-TEST+DOCUMENTATION
+Bổ sung HTTP E2E regression cho inventory movement cursor: trang đầu trả opaque nextCursor, trang kế tiếp không lặp record và malformed cursor vẫn trả 400; không đổi schema hoặc API contract.
+Sources: test:test/admin-contract.e2e-spec.ts, operation:listInventoryMovements, document:25-sprint-2-execution-status.md@1.2.1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F37" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">S2-LEDGER-CURSOR-HTTP-20260907 · 2026-09-07 · API-TEST+DOCUMENTATION
+Bổ sung HTTP E2E regression cho inventory movement cursor: trang đầu trả opaque nextCursor, trang kế tiếp không lặp record và malformed cursor vẫn trả 400; không đổi schema hoặc API contract.
+Sources: test:test/admin-contract.e2e-spec.ts, operation:listInventoryMovements, document:25-sprint-2-execution-status.md@1.2.1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A38" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">D11-SYNC-20260907 · 2026-09-07 · DECISION+DOCUMENTATION
+Đồng bộ D11 từ PROPOSED sang DECIDED theo rule Sprint 2 đã chốt và triển khai: V1 không maker-checker; BRANCH_MANAGER giảm tối đa 10 đơn vị/SKU/lệnh; GLOBAL/OWNER được vượt; reason và audit luôn bắt buộc.
+Sources: decision:D11, document:08-open-decisions.csv, document:25-sprint-2-execution-status.md@1.2.1, source:src/modules/inventory/inventory.service.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B38" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">D11-SYNC-20260907 · 2026-09-07 · DECISION+DOCUMENTATION
+Đồng bộ D11 từ PROPOSED sang DECIDED theo rule Sprint 2 đã chốt và triển khai: V1 không maker-checker; BRANCH_MANAGER giảm tối đa 10 đơn vị/SKU/lệnh; GLOBAL/OWNER được vượt; reason và audit luôn bắt buộc.
+Sources: decision:D11, document:08-open-decisions.csv, document:25-sprint-2-execution-status.md@1.2.1, source:src/modules/inventory/inventory.service.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C38" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">D11-SYNC-20260907 · 2026-09-07 · DECISION+DOCUMENTATION
+Đồng bộ D11 từ PROPOSED sang DECIDED theo rule Sprint 2 đã chốt và triển khai: V1 không maker-checker; BRANCH_MANAGER giảm tối đa 10 đơn vị/SKU/lệnh; GLOBAL/OWNER được vượt; reason và audit luôn bắt buộc.
+Sources: decision:D11, document:08-open-decisions.csv, document:25-sprint-2-execution-status.md@1.2.1, source:src/modules/inventory/inventory.service.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D38" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">D11-SYNC-20260907 · 2026-09-07 · DECISION+DOCUMENTATION
+Đồng bộ D11 từ PROPOSED sang DECIDED theo rule Sprint 2 đã chốt và triển khai: V1 không maker-checker; BRANCH_MANAGER giảm tối đa 10 đơn vị/SKU/lệnh; GLOBAL/OWNER được vượt; reason và audit luôn bắt buộc.
+Sources: decision:D11, document:08-open-decisions.csv, document:25-sprint-2-execution-status.md@1.2.1, source:src/modules/inventory/inventory.service.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E38" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">D11-SYNC-20260907 · 2026-09-07 · DECISION+DOCUMENTATION
+Đồng bộ D11 từ PROPOSED sang DECIDED theo rule Sprint 2 đã chốt và triển khai: V1 không maker-checker; BRANCH_MANAGER giảm tối đa 10 đơn vị/SKU/lệnh; GLOBAL/OWNER được vượt; reason và audit luôn bắt buộc.
+Sources: decision:D11, document:08-open-decisions.csv, document:25-sprint-2-execution-status.md@1.2.1, source:src/modules/inventory/inventory.service.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F38" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">D11-SYNC-20260907 · 2026-09-07 · DECISION+DOCUMENTATION
+Đồng bộ D11 từ PROPOSED sang DECIDED theo rule Sprint 2 đã chốt và triển khai: V1 không maker-checker; BRANCH_MANAGER giảm tối đa 10 đơn vị/SKU/lệnh; GLOBAL/OWNER được vượt; reason và audit luôn bắt buộc.
+Sources: decision:D11, document:08-open-decisions.csv, document:25-sprint-2-execution-status.md@1.2.1, source:src/modules/inventory/inventory.service.ts</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -8107,7 +8261,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7768" uniqueCount="1611">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7781" uniqueCount="1622">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -11568,13 +11722,16 @@
     <t>Approval stock threshold</t>
   </si>
   <si>
-    <t>Cần duyệt khi giảm tồn vượt 10 đơn vị hoặc 5 triệu VND cost</t>
-  </si>
-  <si>
-    <t>Maker-checker cần rule cụ thể</t>
+    <t>V1 không maker-checker; BRANCH_MANAGER giảm tối đa 10 đơn vị mỗi SKU/lệnh; GLOBAL/OWNER được vượt; mọi lần giảm bắt buộc reason và audit</t>
+  </si>
+  <si>
+    <t>Giữ kiểm soát giảm tồn trong V1 mà không kéo approval engine vào sớm</t>
   </si>
   <si>
     <t>Ops+Finance</t>
+  </si>
+  <si>
+    <t>Đã triển khai trong Sprint 2; branch decrease &gt;10 bị từ chối, GLOBAL được vượt; reason và audit bắt buộc.</t>
   </si>
   <si>
     <t>D12</t>
@@ -13124,6 +13281,41 @@
 document:19-admin-api-v1-contract-integration.md@1.2.2
 document:22-repository-split-and-deployment.md@1.4.2
 evidence:local login 200 then auth/me 200 against shared Supabase</t>
+  </si>
+  <si>
+    <t>S2-LEDGER-CURSOR-HTTP-20260907</t>
+  </si>
+  <si>
+    <t>2026-09-07</t>
+  </si>
+  <si>
+    <t>API-TEST+DOCUMENTATION</t>
+  </si>
+  <si>
+    <t>Bổ sung HTTP E2E regression cho inventory movement cursor: trang đầu trả opaque nextCursor, trang kế tiếp không lặp record và malformed cursor vẫn trả 400; không đổi schema hoặc API contract.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test:test/admin-contract.e2e-spec.ts
+operation:listInventoryMovements
+document:25-sprint-2-execution-status.md@1.2.1</t>
+  </si>
+  <si>
+    <t>D11-SYNC-20260907</t>
+  </si>
+  <si>
+    <t>DECISION+DOCUMENTATION</t>
+  </si>
+  <si>
+    <t>Đồng bộ D11 từ PROPOSED sang DECIDED theo rule Sprint 2 đã chốt và triển khai: V1 không maker-checker; BRANCH_MANAGER giảm tối đa 10 đơn vị/SKU/lệnh; GLOBAL/OWNER được vượt; reason và audit luôn bắt buộc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">decision:D11
+document:08-open-decisions.csv
+document:25-sprint-2-execution-status.md@1.2.1
+source:src/modules/inventory/inventory.service.ts</t>
+  </si>
+  <si>
+    <t>Open Decisions: {"ID":"D11"} → Quyết định đề xuất, Tại sao quan trọng, Status, Kết luận review / ghi chú</t>
   </si>
 </sst>
 </file>
@@ -39515,10 +39707,10 @@
       <c r="B12" s="2" t="s">
         <v>1152</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>1153</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="4" t="s">
         <v>1154</v>
       </c>
       <c r="E12" s="2" t="s">
@@ -39527,23 +39719,25 @@
       <c r="F12" s="2" t="s">
         <v>548</v>
       </c>
-      <c r="G12" s="7" t="s">
-        <v>1107</v>
-      </c>
-      <c r="H12" s="2"/>
+      <c r="G12" s="4" t="s">
+        <v>1145</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>1156</v>
+      </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>1159</v>
+        <v>1160</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>1112</v>
@@ -39558,19 +39752,19 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>1160</v>
+        <v>1161</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>1161</v>
+        <v>1162</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>1163</v>
+        <v>1164</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>539</v>
@@ -39582,16 +39776,16 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>1112</v>
@@ -39606,19 +39800,19 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>551</v>
@@ -39630,19 +39824,19 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>1175</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>1176</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>1177</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>1178</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>1174</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>1175</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>1176</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>1177</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>1173</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>555</v>
@@ -39654,19 +39848,19 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>1181</v>
+        <v>1182</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>1182</v>
+        <v>1183</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>539</v>
@@ -39678,19 +39872,19 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>1187</v>
+        <v>1188</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>562</v>
@@ -39702,19 +39896,19 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>1188</v>
+        <v>1189</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>1189</v>
+        <v>1190</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>1191</v>
+        <v>1192</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>568</v>
@@ -39726,16 +39920,16 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>1106</v>
@@ -39750,19 +39944,19 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>1197</v>
+        <v>1198</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>559</v>
@@ -39774,16 +39968,16 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>1205</v>
+        <v>1206</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>1069</v>
@@ -39798,16 +39992,16 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>1208</v>
+        <v>1209</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>1209</v>
+        <v>1210</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>1069</v>
@@ -39822,16 +40016,16 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>1210</v>
+        <v>1211</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>1211</v>
+        <v>1212</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>1212</v>
+        <v>1213</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>1213</v>
+        <v>1214</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>1069</v>
@@ -39846,16 +40040,16 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>1214</v>
+        <v>1215</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>1216</v>
+        <v>1217</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>1217</v>
+        <v>1218</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>1144</v>
@@ -39870,16 +40064,16 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>1218</v>
+        <v>1219</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>1219</v>
+        <v>1220</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>1220</v>
+        <v>1221</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>1221</v>
+        <v>1222</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>1144</v>
@@ -39894,19 +40088,19 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>1223</v>
+        <v>1224</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>1224</v>
+        <v>1225</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>1225</v>
+        <v>1226</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>1187</v>
+        <v>1188</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>544</v>
@@ -39918,19 +40112,19 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>1227</v>
+        <v>1228</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>1229</v>
+        <v>1230</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>559</v>
@@ -39942,19 +40136,19 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>1230</v>
+        <v>1231</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>1232</v>
+        <v>1233</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>1233</v>
+        <v>1234</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>559</v>
@@ -39966,19 +40160,19 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>1235</v>
+        <v>1236</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>1236</v>
+        <v>1237</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>1237</v>
+        <v>1238</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>1239</v>
+        <v>1240</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>555</v>
@@ -39990,19 +40184,19 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>1241</v>
+        <v>1242</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>1242</v>
+        <v>1243</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>555</v>
@@ -40014,16 +40208,16 @@
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>1244</v>
+        <v>1245</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>1245</v>
+        <v>1246</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>1247</v>
+        <v>1248</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>1144</v>
@@ -40039,6 +40233,7 @@
   </sheetData>
   <autoFilter ref="A1:H33"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -40058,22 +40253,22 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>1248</v>
+        <v>1249</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1250</v>
+        <v>1251</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1251</v>
+        <v>1252</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1252</v>
+        <v>1253</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>1046</v>
@@ -40081,1042 +40276,1042 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>1257</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>1258</v>
+        <v>1259</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>1261</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>1262</v>
+        <v>1263</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>1264</v>
+        <v>1265</v>
       </c>
       <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>1267</v>
+        <v>1268</v>
       </c>
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>62</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>1269</v>
+        <v>1270</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>1270</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>1271</v>
+        <v>1272</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>62</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>1272</v>
+        <v>1273</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>1273</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>1274</v>
+        <v>1275</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>62</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>1272</v>
+        <v>1273</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>1275</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>1276</v>
+        <v>1277</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>62</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>1277</v>
+        <v>1278</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>1278</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>1279</v>
+        <v>1280</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>62</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>1272</v>
+        <v>1273</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>1281</v>
+        <v>1282</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>62</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>1272</v>
+        <v>1273</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>1282</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>117</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>1285</v>
+        <v>1286</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>1286</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>1287</v>
+        <v>1288</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>117</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>1288</v>
+        <v>1289</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>1289</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>1290</v>
+        <v>1291</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>131</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>1291</v>
+        <v>1292</v>
       </c>
       <c r="G14" s="2"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>1292</v>
+        <v>1293</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>131</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>1293</v>
+        <v>1294</v>
       </c>
       <c r="G15" s="2"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>1294</v>
+        <v>1295</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>131</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>1295</v>
+        <v>1296</v>
       </c>
       <c r="G16" s="2"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>1296</v>
+        <v>1297</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>131</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>1293</v>
+        <v>1294</v>
       </c>
       <c r="G17" s="2"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>1297</v>
+        <v>1298</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>131</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>1298</v>
+        <v>1299</v>
       </c>
       <c r="G18" s="2"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>1299</v>
+        <v>1300</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>131</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>1293</v>
+        <v>1294</v>
       </c>
       <c r="G19" s="2"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>1300</v>
+        <v>1301</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>131</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>1301</v>
+        <v>1302</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>1293</v>
+        <v>1294</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>1302</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>1303</v>
+        <v>1304</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>131</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>1304</v>
+        <v>1305</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>1305</v>
+        <v>1306</v>
       </c>
       <c r="G21" s="2"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>1306</v>
+        <v>1307</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>131</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>1307</v>
+        <v>1308</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>1308</v>
+        <v>1309</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>1309</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>1310</v>
+        <v>1311</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>202</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="G23" s="2"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>1312</v>
+        <v>1313</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>202</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>1313</v>
+        <v>1314</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>1315</v>
+        <v>1316</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>202</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>1316</v>
+        <v>1317</v>
       </c>
       <c r="G25" s="2"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>1317</v>
+        <v>1318</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>202</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>1316</v>
+        <v>1317</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>1318</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>230</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>1320</v>
+        <v>1321</v>
       </c>
       <c r="G27" s="2"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>1321</v>
+        <v>1322</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>230</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>1322</v>
+        <v>1323</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>1324</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>1325</v>
+        <v>1326</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>230</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>1327</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>1328</v>
+        <v>1329</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>547</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>541</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>541</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>1342</v>
+        <v>1343</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>1343</v>
+        <v>1344</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>541</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>1344</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>302</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>1347</v>
+        <v>1348</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>1348</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>1349</v>
+        <v>1350</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>302</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>1350</v>
+        <v>1351</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>1351</v>
+        <v>1352</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>1352</v>
+        <v>1353</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>1353</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>1354</v>
+        <v>1355</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>302</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>1355</v>
+        <v>1356</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>302</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>326</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>1363</v>
+        <v>1364</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>326</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>1365</v>
+        <v>1366</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>1366</v>
+        <v>1367</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>326</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>1370</v>
+        <v>1371</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>1371</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>1372</v>
+        <v>1373</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>326</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>1373</v>
+        <v>1374</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>1375</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>1376</v>
+        <v>1377</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>351</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>1377</v>
+        <v>1378</v>
       </c>
       <c r="G42" s="2"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>1378</v>
+        <v>1379</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>351</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>1379</v>
+        <v>1380</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>1380</v>
+        <v>1381</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>1381</v>
+        <v>1382</v>
       </c>
       <c r="G43" s="2"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>1382</v>
+        <v>1383</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>351</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>1383</v>
+        <v>1384</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>1380</v>
+        <v>1381</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>1381</v>
+        <v>1382</v>
       </c>
       <c r="G44" s="2"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>1384</v>
+        <v>1385</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>351</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>1385</v>
+        <v>1386</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>1380</v>
+        <v>1381</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>1381</v>
+        <v>1382</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>1386</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>1387</v>
+        <v>1388</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>351</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>1388</v>
+        <v>1389</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>1355</v>
+        <v>1356</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>1389</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>1390</v>
+        <v>1391</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>384</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>1391</v>
+        <v>1392</v>
       </c>
       <c r="G47" s="2"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>1392</v>
+        <v>1393</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>384</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>1351</v>
+        <v>1352</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>614</v>
@@ -41125,342 +41320,342 @@
         <v>117</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>1393</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>1394</v>
+        <v>1395</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>384</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>1395</v>
+        <v>1396</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>1396</v>
+        <v>1397</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>1397</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>1398</v>
+        <v>1399</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>384</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>1399</v>
+        <v>1400</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>1380</v>
+        <v>1381</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>1381</v>
+        <v>1382</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>1400</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>1401</v>
+        <v>1402</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>403</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>1402</v>
+        <v>1403</v>
       </c>
       <c r="G51" s="2"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>1403</v>
+        <v>1404</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>403</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>1402</v>
+        <v>1403</v>
       </c>
       <c r="G52" s="2"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>1404</v>
+        <v>1405</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>454</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>1405</v>
+        <v>1406</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>1406</v>
+        <v>1407</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>1407</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>1408</v>
+        <v>1409</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>454</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>1409</v>
+        <v>1410</v>
       </c>
       <c r="G54" s="2"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>1410</v>
+        <v>1411</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>454</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>1411</v>
+        <v>1412</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>1412</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>1413</v>
+        <v>1414</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>422</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>1414</v>
+        <v>1415</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>1415</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>1416</v>
+        <v>1417</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>1417</v>
+        <v>1418</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>1418</v>
+        <v>1419</v>
       </c>
       <c r="G57" s="2"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>1419</v>
+        <v>1420</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>1417</v>
+        <v>1418</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>1420</v>
+        <v>1421</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>1421</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>1422</v>
+        <v>1423</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>1417</v>
+        <v>1418</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>614</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>1423</v>
+        <v>1424</v>
       </c>
       <c r="G59" s="2"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>1424</v>
+        <v>1425</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>1417</v>
+        <v>1418</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>1425</v>
+        <v>1426</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>1426</v>
+        <v>1427</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>1427</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>1428</v>
+        <v>1429</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>107</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>1429</v>
+        <v>1430</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>1430</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>1431</v>
+        <v>1432</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>107</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>1395</v>
+        <v>1396</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>1432</v>
+        <v>1433</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>1433</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>1434</v>
+        <v>1435</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>435</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>581</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>1435</v>
+        <v>1436</v>
       </c>
     </row>
   </sheetData>
@@ -41472,7 +41667,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -41485,722 +41680,762 @@
   <sheetData>
     <row r="1" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>1438</v>
+        <v>1439</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>1439</v>
+        <v>1440</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>1440</v>
+        <v>1441</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>1441</v>
+        <v>1442</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>1442</v>
+        <v>1443</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>1443</v>
+        <v>1444</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>1444</v>
+        <v>1445</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>1446</v>
+        <v>1447</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>1447</v>
+        <v>1448</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>1448</v>
+        <v>1449</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>1449</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>1450</v>
+        <v>1451</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>1451</v>
+        <v>1452</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>1452</v>
+        <v>1453</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>1453</v>
+        <v>1454</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>1454</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>1455</v>
+        <v>1456</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>1446</v>
+        <v>1447</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>1456</v>
+        <v>1457</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>1457</v>
+        <v>1458</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>1458</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>1459</v>
+        <v>1460</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>1460</v>
+        <v>1461</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>1461</v>
+        <v>1462</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>1462</v>
+        <v>1463</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>1463</v>
+        <v>1464</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>1464</v>
+        <v>1465</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>1465</v>
+        <v>1466</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>1466</v>
+        <v>1467</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>1467</v>
+        <v>1468</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
+        <v>1470</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>1446</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>1471</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>1472</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>1473</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>1469</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>1445</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>1470</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>1471</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>1472</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>1468</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>1446</v>
+        <v>1447</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>1473</v>
+        <v>1474</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>1474</v>
+        <v>1475</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>1475</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>1476</v>
+        <v>1477</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>1477</v>
+        <v>1478</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>1478</v>
+        <v>1479</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>1479</v>
+        <v>1480</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>1480</v>
+        <v>1481</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>1481</v>
+        <v>1482</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>1477</v>
+        <v>1478</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>1482</v>
+        <v>1483</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>1483</v>
+        <v>1484</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>1484</v>
+        <v>1485</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>1485</v>
+        <v>1486</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>1486</v>
+        <v>1487</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>1487</v>
+        <v>1488</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>1488</v>
+        <v>1489</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>1489</v>
+        <v>1490</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>1490</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>1491</v>
+        <v>1492</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>1486</v>
+        <v>1487</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>1492</v>
+        <v>1493</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>1493</v>
+        <v>1494</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>1494</v>
+        <v>1495</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>1495</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>1496</v>
+        <v>1497</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>1497</v>
+        <v>1498</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>1498</v>
+        <v>1499</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>1499</v>
+        <v>1500</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>1500</v>
+        <v>1501</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>1501</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>1502</v>
+        <v>1503</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>1503</v>
+        <v>1504</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>1482</v>
+        <v>1483</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>1504</v>
+        <v>1505</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>1505</v>
+        <v>1506</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>1506</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>1507</v>
+        <v>1508</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>1503</v>
+        <v>1504</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>1508</v>
+        <v>1509</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>1509</v>
+        <v>1510</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>1510</v>
+        <v>1511</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>1511</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>1512</v>
+        <v>1513</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>1503</v>
+        <v>1504</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>1513</v>
+        <v>1514</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>1514</v>
+        <v>1515</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>1515</v>
+        <v>1516</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>1516</v>
+        <v>1517</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>1517</v>
+        <v>1518</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>1503</v>
+        <v>1504</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>1518</v>
+        <v>1519</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>1519</v>
+        <v>1520</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>1521</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>1522</v>
+        <v>1523</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>1503</v>
+        <v>1504</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>1523</v>
+        <v>1524</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>1524</v>
+        <v>1525</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>1525</v>
+        <v>1526</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>1526</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>1527</v>
+        <v>1528</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>1528</v>
+        <v>1529</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>1529</v>
+        <v>1530</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>1530</v>
+        <v>1531</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>1531</v>
+        <v>1532</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>1532</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>1533</v>
+        <v>1534</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>1528</v>
+        <v>1529</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>1534</v>
+        <v>1535</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>1535</v>
+        <v>1536</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>1536</v>
+        <v>1537</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>1537</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>1538</v>
+        <v>1539</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>1540</v>
+        <v>1541</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>1541</v>
+        <v>1542</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>1542</v>
+        <v>1543</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>1543</v>
+        <v>1544</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>1544</v>
+        <v>1545</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>1545</v>
+        <v>1546</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>1546</v>
+        <v>1547</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>1547</v>
+        <v>1548</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>1548</v>
+        <v>1549</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>1549</v>
+        <v>1550</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>1551</v>
+        <v>1552</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>1552</v>
+        <v>1553</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>1553</v>
+        <v>1554</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>1554</v>
+        <v>1555</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>1555</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>1556</v>
+        <v>1557</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>1557</v>
+        <v>1558</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>1558</v>
+        <v>1559</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>1559</v>
+        <v>1560</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>1560</v>
+        <v>1561</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>1561</v>
+        <v>1562</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>1562</v>
+        <v>1563</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>1563</v>
+        <v>1564</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>1564</v>
+        <v>1565</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>1566</v>
+        <v>1567</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>1567</v>
+        <v>1568</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>1568</v>
+        <v>1569</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>1569</v>
+        <v>1570</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>1570</v>
+        <v>1571</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>1571</v>
+        <v>1572</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>1572</v>
+        <v>1573</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>1573</v>
+        <v>1574</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>1575</v>
+        <v>1576</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>1576</v>
+        <v>1577</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>1577</v>
+        <v>1578</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>1578</v>
+        <v>1579</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>1579</v>
+        <v>1580</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>1580</v>
+        <v>1581</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>1582</v>
+        <v>1583</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>1583</v>
+        <v>1584</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>1584</v>
+        <v>1585</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>1589</v>
+        <v>1590</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>1590</v>
+        <v>1591</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>1592</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>1593</v>
+        <v>1594</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>1594</v>
+        <v>1595</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>1595</v>
+        <v>1596</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>1596</v>
+        <v>1597</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>1598</v>
+        <v>1599</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>1600</v>
+        <v>1601</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>1601</v>
+        <v>1602</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>1604</v>
+        <v>1605</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>1606</v>
+        <v>1607</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>1607</v>
+        <v>1608</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>1468</v>
+        <v>1469</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>1613</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>1614</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>1615</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>1616</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>1469</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>1617</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>1613</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>1618</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>1619</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>1620</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>1621</v>
       </c>
     </row>
   </sheetData>
@@ -42256,7 +42491,7 @@
         <v>538</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>1436</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -42288,7 +42523,7 @@
         <v>801</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -42320,7 +42555,7 @@
         <v>801</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -42352,7 +42587,7 @@
         <v>801</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -42384,7 +42619,7 @@
         <v>801</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -42416,7 +42651,7 @@
         <v>801</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -42448,7 +42683,7 @@
         <v>801</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -42480,7 +42715,7 @@
         <v>801</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -42512,7 +42747,7 @@
         <v>801</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -42544,7 +42779,7 @@
         <v>801</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -42576,7 +42811,7 @@
         <v>801</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add admin shipping consultation feature with DTOs and service logic
- Introduced AdminShippingConsultationDto, AdminShippingConsultationListDto, and AdminShippingConsultationQueryDto for handling shipping consultations.
- Implemented listShippingConsultations method in CheckoutService to retrieve consultations based on user permissions and filters.
- Added ReservationExpiryController and ReservationExpiryService to manage reservation expiry jobs with cron-like functionality.
- Enhanced CheckoutService with new methods for handling shipping consultations and improved error handling.
- Created unit and integration tests for new features, ensuring proper functionality and concurrency handling.
- Updated existing tests to reflect changes in error messages and validation.
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -6266,6 +6266,78 @@
         </r>
       </text>
     </comment>
+    <comment ref="A37" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBSEC-20260909-PUBLIC-RLS-COMPLETE · 2026-09-09 · DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION
+Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.
+Sources: migration:20260909010000_harden_all_public_tables_rls, test:test/database-security.integration-spec.ts, decision:D46, document:03-database-v1.md@2.6.0, document:25-sprint-2-execution-status.md@1.3.1, evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B37" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBSEC-20260909-PUBLIC-RLS-COMPLETE · 2026-09-09 · DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION
+Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.
+Sources: migration:20260909010000_harden_all_public_tables_rls, test:test/database-security.integration-spec.ts, decision:D46, document:03-database-v1.md@2.6.0, document:25-sprint-2-execution-status.md@1.3.1, evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C37" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBSEC-20260909-PUBLIC-RLS-COMPLETE · 2026-09-09 · DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION
+Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.
+Sources: migration:20260909010000_harden_all_public_tables_rls, test:test/database-security.integration-spec.ts, decision:D46, document:03-database-v1.md@2.6.0, document:25-sprint-2-execution-status.md@1.3.1, evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D37" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBSEC-20260909-PUBLIC-RLS-COMPLETE · 2026-09-09 · DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION
+Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.
+Sources: migration:20260909010000_harden_all_public_tables_rls, test:test/database-security.integration-spec.ts, decision:D46, document:03-database-v1.md@2.6.0, document:25-sprint-2-execution-status.md@1.3.1, evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E37" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBSEC-20260909-PUBLIC-RLS-COMPLETE · 2026-09-09 · DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION
+Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.
+Sources: migration:20260909010000_harden_all_public_tables_rls, test:test/database-security.integration-spec.ts, decision:D46, document:03-database-v1.md@2.6.0, document:25-sprint-2-execution-status.md@1.3.1, evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F37" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBSEC-20260909-PUBLIC-RLS-COMPLETE · 2026-09-09 · DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION
+Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.
+Sources: migration:20260909010000_harden_all_public_tables_rls, test:test/database-security.integration-spec.ts, decision:D46, document:03-database-v1.md@2.6.0, document:25-sprint-2-execution-status.md@1.3.1, evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G37" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBSEC-20260909-PUBLIC-RLS-COMPLETE · 2026-09-09 · DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION
+Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.
+Sources: migration:20260909010000_harden_all_public_tables_rls, test:test/database-security.integration-spec.ts, decision:D46, document:03-database-v1.md@2.6.0, document:25-sprint-2-execution-status.md@1.3.1, evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H37" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBSEC-20260909-PUBLIC-RLS-COMPLETE · 2026-09-09 · DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION
+Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.
+Sources: migration:20260909010000_harden_all_public_tables_rls, test:test/database-security.integration-spec.ts, decision:D46, document:03-database-v1.md@2.6.0, document:25-sprint-2-execution-status.md@1.3.1, evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -9103,6 +9175,222 @@
         </r>
       </text>
     </comment>
+    <comment ref="A47" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260908-CHECKOUT-CONSULTATION-ROUNDTRIP · 2026-09-08 · CHECKOUT+OPENAPI+STOREFRONT+ADMIN
+Không đổi schema; thêm API Admin list manual consultation theo branch scope, API Client đọc lại owned quote và request flag; cả hai FE dùng SDK sinh từ OpenAPI.
+Sources: operation:listAdminShippingConsultations/updateAdminManualShippingQuote, operation:getGuestCheckoutQuote/getAccountCheckoutQuote/quoteGuestCheckout/quoteAccountCheckout, test:src/modules/checkout/checkout.service.spec.ts, contract:document/api/admin/checkout.yaml/document/api/storefront/checkout.yaml, document:06-rules-and-state-machines.md@1.4.0, document:28-sprint-3-execution-status.md@1.7.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B47" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260908-CHECKOUT-CONSULTATION-ROUNDTRIP · 2026-09-08 · CHECKOUT+OPENAPI+STOREFRONT+ADMIN
+Không đổi schema; thêm API Admin list manual consultation theo branch scope, API Client đọc lại owned quote và request flag; cả hai FE dùng SDK sinh từ OpenAPI.
+Sources: operation:listAdminShippingConsultations/updateAdminManualShippingQuote, operation:getGuestCheckoutQuote/getAccountCheckoutQuote/quoteGuestCheckout/quoteAccountCheckout, test:src/modules/checkout/checkout.service.spec.ts, contract:document/api/admin/checkout.yaml/document/api/storefront/checkout.yaml, document:06-rules-and-state-machines.md@1.4.0, document:28-sprint-3-execution-status.md@1.7.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C47" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260908-CHECKOUT-CONSULTATION-ROUNDTRIP · 2026-09-08 · CHECKOUT+OPENAPI+STOREFRONT+ADMIN
+Không đổi schema; thêm API Admin list manual consultation theo branch scope, API Client đọc lại owned quote và request flag; cả hai FE dùng SDK sinh từ OpenAPI.
+Sources: operation:listAdminShippingConsultations/updateAdminManualShippingQuote, operation:getGuestCheckoutQuote/getAccountCheckoutQuote/quoteGuestCheckout/quoteAccountCheckout, test:src/modules/checkout/checkout.service.spec.ts, contract:document/api/admin/checkout.yaml/document/api/storefront/checkout.yaml, document:06-rules-and-state-machines.md@1.4.0, document:28-sprint-3-execution-status.md@1.7.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D47" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260908-CHECKOUT-CONSULTATION-ROUNDTRIP · 2026-09-08 · CHECKOUT+OPENAPI+STOREFRONT+ADMIN
+Không đổi schema; thêm API Admin list manual consultation theo branch scope, API Client đọc lại owned quote và request flag; cả hai FE dùng SDK sinh từ OpenAPI.
+Sources: operation:listAdminShippingConsultations/updateAdminManualShippingQuote, operation:getGuestCheckoutQuote/getAccountCheckoutQuote/quoteGuestCheckout/quoteAccountCheckout, test:src/modules/checkout/checkout.service.spec.ts, contract:document/api/admin/checkout.yaml/document/api/storefront/checkout.yaml, document:06-rules-and-state-machines.md@1.4.0, document:28-sprint-3-execution-status.md@1.7.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E47" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260908-CHECKOUT-CONSULTATION-ROUNDTRIP · 2026-09-08 · CHECKOUT+OPENAPI+STOREFRONT+ADMIN
+Không đổi schema; thêm API Admin list manual consultation theo branch scope, API Client đọc lại owned quote và request flag; cả hai FE dùng SDK sinh từ OpenAPI.
+Sources: operation:listAdminShippingConsultations/updateAdminManualShippingQuote, operation:getGuestCheckoutQuote/getAccountCheckoutQuote/quoteGuestCheckout/quoteAccountCheckout, test:src/modules/checkout/checkout.service.spec.ts, contract:document/api/admin/checkout.yaml/document/api/storefront/checkout.yaml, document:06-rules-and-state-machines.md@1.4.0, document:28-sprint-3-execution-status.md@1.7.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F47" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260908-CHECKOUT-CONSULTATION-ROUNDTRIP · 2026-09-08 · CHECKOUT+OPENAPI+STOREFRONT+ADMIN
+Không đổi schema; thêm API Admin list manual consultation theo branch scope, API Client đọc lại owned quote và request flag; cả hai FE dùng SDK sinh từ OpenAPI.
+Sources: operation:listAdminShippingConsultations/updateAdminManualShippingQuote, operation:getGuestCheckoutQuote/getAccountCheckoutQuote/quoteGuestCheckout/quoteAccountCheckout, test:src/modules/checkout/checkout.service.spec.ts, contract:document/api/admin/checkout.yaml/document/api/storefront/checkout.yaml, document:06-rules-and-state-machines.md@1.4.0, document:28-sprint-3-execution-status.md@1.7.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A48" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260908-RESERVATION-EXPIRY-WORKER · 2026-09-08 · CHECKOUT+INVENTORY+AUDIT+OPERATIONS+DOCUMENTATION
+Không đổi schema; thêm expiry worker batch-safe, secured internal endpoint và bộ cấu hình Supabase Cron/pg_net/Vault.
+Sources: operation:ReservationExpiryService.run, endpoint:GET /api/v1/internal/jobs/reservations/expire, script:scripts/configure-reservation-expiry-cron.cjs, test:src/modules/checkout/reservation-expiry.service.spec.ts/src/modules/checkout/reservation-expiry.controller.spec.ts, document:06-rules-and-state-machines.md@1.5.0, document:28-sprint-3-execution-status.md@1.8.0, document:29-reservation-expiry-worker-runbook.md@1.0.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B48" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260908-RESERVATION-EXPIRY-WORKER · 2026-09-08 · CHECKOUT+INVENTORY+AUDIT+OPERATIONS+DOCUMENTATION
+Không đổi schema; thêm expiry worker batch-safe, secured internal endpoint và bộ cấu hình Supabase Cron/pg_net/Vault.
+Sources: operation:ReservationExpiryService.run, endpoint:GET /api/v1/internal/jobs/reservations/expire, script:scripts/configure-reservation-expiry-cron.cjs, test:src/modules/checkout/reservation-expiry.service.spec.ts/src/modules/checkout/reservation-expiry.controller.spec.ts, document:06-rules-and-state-machines.md@1.5.0, document:28-sprint-3-execution-status.md@1.8.0, document:29-reservation-expiry-worker-runbook.md@1.0.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C48" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260908-RESERVATION-EXPIRY-WORKER · 2026-09-08 · CHECKOUT+INVENTORY+AUDIT+OPERATIONS+DOCUMENTATION
+Không đổi schema; thêm expiry worker batch-safe, secured internal endpoint và bộ cấu hình Supabase Cron/pg_net/Vault.
+Sources: operation:ReservationExpiryService.run, endpoint:GET /api/v1/internal/jobs/reservations/expire, script:scripts/configure-reservation-expiry-cron.cjs, test:src/modules/checkout/reservation-expiry.service.spec.ts/src/modules/checkout/reservation-expiry.controller.spec.ts, document:06-rules-and-state-machines.md@1.5.0, document:28-sprint-3-execution-status.md@1.8.0, document:29-reservation-expiry-worker-runbook.md@1.0.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D48" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260908-RESERVATION-EXPIRY-WORKER · 2026-09-08 · CHECKOUT+INVENTORY+AUDIT+OPERATIONS+DOCUMENTATION
+Không đổi schema; thêm expiry worker batch-safe, secured internal endpoint và bộ cấu hình Supabase Cron/pg_net/Vault.
+Sources: operation:ReservationExpiryService.run, endpoint:GET /api/v1/internal/jobs/reservations/expire, script:scripts/configure-reservation-expiry-cron.cjs, test:src/modules/checkout/reservation-expiry.service.spec.ts/src/modules/checkout/reservation-expiry.controller.spec.ts, document:06-rules-and-state-machines.md@1.5.0, document:28-sprint-3-execution-status.md@1.8.0, document:29-reservation-expiry-worker-runbook.md@1.0.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E48" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260908-RESERVATION-EXPIRY-WORKER · 2026-09-08 · CHECKOUT+INVENTORY+AUDIT+OPERATIONS+DOCUMENTATION
+Không đổi schema; thêm expiry worker batch-safe, secured internal endpoint và bộ cấu hình Supabase Cron/pg_net/Vault.
+Sources: operation:ReservationExpiryService.run, endpoint:GET /api/v1/internal/jobs/reservations/expire, script:scripts/configure-reservation-expiry-cron.cjs, test:src/modules/checkout/reservation-expiry.service.spec.ts/src/modules/checkout/reservation-expiry.controller.spec.ts, document:06-rules-and-state-machines.md@1.5.0, document:28-sprint-3-execution-status.md@1.8.0, document:29-reservation-expiry-worker-runbook.md@1.0.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F48" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260908-RESERVATION-EXPIRY-WORKER · 2026-09-08 · CHECKOUT+INVENTORY+AUDIT+OPERATIONS+DOCUMENTATION
+Không đổi schema; thêm expiry worker batch-safe, secured internal endpoint và bộ cấu hình Supabase Cron/pg_net/Vault.
+Sources: operation:ReservationExpiryService.run, endpoint:GET /api/v1/internal/jobs/reservations/expire, script:scripts/configure-reservation-expiry-cron.cjs, test:src/modules/checkout/reservation-expiry.service.spec.ts/src/modules/checkout/reservation-expiry.controller.spec.ts, document:06-rules-and-state-machines.md@1.5.0, document:28-sprint-3-execution-status.md@1.8.0, document:29-reservation-expiry-worker-runbook.md@1.0.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A49" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260909-VIETNAMESE-ERROR-MESSAGES · 2026-09-09 · API+OPENAPI+ADMIN+STOREFRONT+DOCUMENTATION
+Không đổi schema; chuẩn hóa toàn bộ message và details[].message lỗi HTTP sang tiếng Việt tại global exception filter, giữ nguyên code máy và error envelope v1.
+Sources: source:src/common/exceptions/client-error-message.vi.ts, source:src/common/filters/http-exception.filter.ts, test:src/common/exceptions/client-error-message.vi.spec.ts/src/common/filters/http-exception.filter.spec.ts/test/admin-contract.e2e-spec.ts, contract:document/api/openapi-v1.yaml, document:19-admin-api-v1-contract-integration.md@1.3.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B49" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260909-VIETNAMESE-ERROR-MESSAGES · 2026-09-09 · API+OPENAPI+ADMIN+STOREFRONT+DOCUMENTATION
+Không đổi schema; chuẩn hóa toàn bộ message và details[].message lỗi HTTP sang tiếng Việt tại global exception filter, giữ nguyên code máy và error envelope v1.
+Sources: source:src/common/exceptions/client-error-message.vi.ts, source:src/common/filters/http-exception.filter.ts, test:src/common/exceptions/client-error-message.vi.spec.ts/src/common/filters/http-exception.filter.spec.ts/test/admin-contract.e2e-spec.ts, contract:document/api/openapi-v1.yaml, document:19-admin-api-v1-contract-integration.md@1.3.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C49" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260909-VIETNAMESE-ERROR-MESSAGES · 2026-09-09 · API+OPENAPI+ADMIN+STOREFRONT+DOCUMENTATION
+Không đổi schema; chuẩn hóa toàn bộ message và details[].message lỗi HTTP sang tiếng Việt tại global exception filter, giữ nguyên code máy và error envelope v1.
+Sources: source:src/common/exceptions/client-error-message.vi.ts, source:src/common/filters/http-exception.filter.ts, test:src/common/exceptions/client-error-message.vi.spec.ts/src/common/filters/http-exception.filter.spec.ts/test/admin-contract.e2e-spec.ts, contract:document/api/openapi-v1.yaml, document:19-admin-api-v1-contract-integration.md@1.3.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D49" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260909-VIETNAMESE-ERROR-MESSAGES · 2026-09-09 · API+OPENAPI+ADMIN+STOREFRONT+DOCUMENTATION
+Không đổi schema; chuẩn hóa toàn bộ message và details[].message lỗi HTTP sang tiếng Việt tại global exception filter, giữ nguyên code máy và error envelope v1.
+Sources: source:src/common/exceptions/client-error-message.vi.ts, source:src/common/filters/http-exception.filter.ts, test:src/common/exceptions/client-error-message.vi.spec.ts/src/common/filters/http-exception.filter.spec.ts/test/admin-contract.e2e-spec.ts, contract:document/api/openapi-v1.yaml, document:19-admin-api-v1-contract-integration.md@1.3.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E49" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260909-VIETNAMESE-ERROR-MESSAGES · 2026-09-09 · API+OPENAPI+ADMIN+STOREFRONT+DOCUMENTATION
+Không đổi schema; chuẩn hóa toàn bộ message và details[].message lỗi HTTP sang tiếng Việt tại global exception filter, giữ nguyên code máy và error envelope v1.
+Sources: source:src/common/exceptions/client-error-message.vi.ts, source:src/common/filters/http-exception.filter.ts, test:src/common/exceptions/client-error-message.vi.spec.ts/src/common/filters/http-exception.filter.spec.ts/test/admin-contract.e2e-spec.ts, contract:document/api/openapi-v1.yaml, document:19-admin-api-v1-contract-integration.md@1.3.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F49" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260909-VIETNAMESE-ERROR-MESSAGES · 2026-09-09 · API+OPENAPI+ADMIN+STOREFRONT+DOCUMENTATION
+Không đổi schema; chuẩn hóa toàn bộ message và details[].message lỗi HTTP sang tiếng Việt tại global exception filter, giữ nguyên code máy và error envelope v1.
+Sources: source:src/common/exceptions/client-error-message.vi.ts, source:src/common/filters/http-exception.filter.ts, test:src/common/exceptions/client-error-message.vi.spec.ts/src/common/filters/http-exception.filter.spec.ts/test/admin-contract.e2e-spec.ts, contract:document/api/openapi-v1.yaml, document:19-admin-api-v1-contract-integration.md@1.3.0</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A50" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBSEC-20260909-PUBLIC-RLS-COMPLETE · 2026-09-09 · DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION
+Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.
+Sources: migration:20260909010000_harden_all_public_tables_rls, test:test/database-security.integration-spec.ts, decision:D46, document:03-database-v1.md@2.6.0, document:25-sprint-2-execution-status.md@1.3.1, evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B50" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBSEC-20260909-PUBLIC-RLS-COMPLETE · 2026-09-09 · DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION
+Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.
+Sources: migration:20260909010000_harden_all_public_tables_rls, test:test/database-security.integration-spec.ts, decision:D46, document:03-database-v1.md@2.6.0, document:25-sprint-2-execution-status.md@1.3.1, evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C50" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBSEC-20260909-PUBLIC-RLS-COMPLETE · 2026-09-09 · DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION
+Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.
+Sources: migration:20260909010000_harden_all_public_tables_rls, test:test/database-security.integration-spec.ts, decision:D46, document:03-database-v1.md@2.6.0, document:25-sprint-2-execution-status.md@1.3.1, evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D50" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBSEC-20260909-PUBLIC-RLS-COMPLETE · 2026-09-09 · DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION
+Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.
+Sources: migration:20260909010000_harden_all_public_tables_rls, test:test/database-security.integration-spec.ts, decision:D46, document:03-database-v1.md@2.6.0, document:25-sprint-2-execution-status.md@1.3.1, evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E50" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBSEC-20260909-PUBLIC-RLS-COMPLETE · 2026-09-09 · DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION
+Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.
+Sources: migration:20260909010000_harden_all_public_tables_rls, test:test/database-security.integration-spec.ts, decision:D46, document:03-database-v1.md@2.6.0, document:25-sprint-2-execution-status.md@1.3.1, evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F50" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">DBSEC-20260909-PUBLIC-RLS-COMPLETE · 2026-09-09 · DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION
+Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.
+Sources: migration:20260909010000_harden_all_public_tables_rls, test:test/database-security.integration-spec.ts, decision:D46, document:03-database-v1.md@2.6.0, document:25-sprint-2-execution-status.md@1.3.1, evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -10108,7 +10396,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7907" uniqueCount="1715">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7939" uniqueCount="1739">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -13978,6 +14266,24 @@
   </si>
   <si>
     <t>Branch selection thủ công tắt; manual external bắt buộc fee/ETA/provider/note và customer confirm lại.</t>
+  </si>
+  <si>
+    <t>D46</t>
+  </si>
+  <si>
+    <t>Supabase Data API boundary</t>
+  </si>
+  <si>
+    <t>V1 chỉ truy cập dữ liệu qua NestJS/Prisma; mọi public base table bật RLS deny-by-default; anon/authenticated không có table, sequence hoặc application-function privilege; không FORCE RLS cho owner connection</t>
+  </si>
+  <si>
+    <t>Đóng truy cập PostgREST trực tiếp nhưng vẫn giữ Prisma migration/runtime; Data API tương lai phải opt-in theo contract và có policy test</t>
+  </si>
+  <si>
+    <t>Security+Tech</t>
+  </si>
+  <si>
+    <t>Live audit trước migration: 35/35 bảng nghiệp vụ đã bật RLS và không cấp anon/authenticated; chỉ _prisma_migrations thiếu RLS. Migration mới bao phủ toàn bộ public base table và thu hồi EXECUTE trực tiếp trên application-owned function.</t>
   </si>
   <si>
     <t>Permission code</t>
@@ -15512,6 +15818,80 @@
   </si>
   <si>
     <t>Tables: {"Tên bảng":"checkout_sessions"} → Ý nghĩa, Unique / CHECK, Các cột chính</t>
+  </si>
+  <si>
+    <t>API-20260908-CHECKOUT-CONSULTATION-ROUNDTRIP</t>
+  </si>
+  <si>
+    <t>CHECKOUT+OPENAPI+STOREFRONT+ADMIN</t>
+  </si>
+  <si>
+    <t>Không đổi schema; thêm API Admin list manual consultation theo branch scope, API Client đọc lại owned quote và request flag; cả hai FE dùng SDK sinh từ OpenAPI.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">operation:listAdminShippingConsultations/updateAdminManualShippingQuote
+operation:getGuestCheckoutQuote/getAccountCheckoutQuote/quoteGuestCheckout/quoteAccountCheckout
+test:src/modules/checkout/checkout.service.spec.ts
+contract:document/api/admin/checkout.yaml/document/api/storefront/checkout.yaml
+document:06-rules-and-state-machines.md@1.4.0
+document:28-sprint-3-execution-status.md@1.7.0</t>
+  </si>
+  <si>
+    <t>API-20260908-RESERVATION-EXPIRY-WORKER</t>
+  </si>
+  <si>
+    <t>CHECKOUT+INVENTORY+AUDIT+OPERATIONS+DOCUMENTATION</t>
+  </si>
+  <si>
+    <t>Không đổi schema; thêm expiry worker batch-safe, secured internal endpoint và bộ cấu hình Supabase Cron/pg_net/Vault.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">operation:ReservationExpiryService.run
+endpoint:GET /api/v1/internal/jobs/reservations/expire
+script:scripts/configure-reservation-expiry-cron.cjs
+test:src/modules/checkout/reservation-expiry.service.spec.ts/src/modules/checkout/reservation-expiry.controller.spec.ts
+document:06-rules-and-state-machines.md@1.5.0
+document:28-sprint-3-execution-status.md@1.8.0
+document:29-reservation-expiry-worker-runbook.md@1.0.0</t>
+  </si>
+  <si>
+    <t>API-20260909-VIETNAMESE-ERROR-MESSAGES</t>
+  </si>
+  <si>
+    <t>2026-09-09</t>
+  </si>
+  <si>
+    <t>API+OPENAPI+ADMIN+STOREFRONT+DOCUMENTATION</t>
+  </si>
+  <si>
+    <t>Không đổi schema; chuẩn hóa toàn bộ message và details[].message lỗi HTTP sang tiếng Việt tại global exception filter, giữ nguyên code máy và error envelope v1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">source:src/common/exceptions/client-error-message.vi.ts
+source:src/common/filters/http-exception.filter.ts
+test:src/common/exceptions/client-error-message.vi.spec.ts/src/common/filters/http-exception.filter.spec.ts/test/admin-contract.e2e-spec.ts
+contract:document/api/openapi-v1.yaml
+document:19-admin-api-v1-contract-integration.md@1.3.0</t>
+  </si>
+  <si>
+    <t>DBSEC-20260909-PUBLIC-RLS-COMPLETE</t>
+  </si>
+  <si>
+    <t>DATABASE+SUPABASE+SECURITY+TEST+DOCUMENTATION</t>
+  </si>
+  <si>
+    <t>Không đổi mô hình nghiệp vụ; bật RLS deny-by-default cho mọi public base table kể cả _prisma_migrations, thu hồi quyền Data API hiện tại và khóa default privilege của table, sequence, application-owned function.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">migration:20260909010000_harden_all_public_tables_rls
+test:test/database-security.integration-spec.ts
+decision:D46
+document:03-database-v1.md@2.6.0
+document:25-sprint-2-execution-status.md@1.3.1
+evidence:live Supabase public-schema RLS and privilege audit 2026-09-09</t>
+  </si>
+  <si>
+    <t>Open Decisions: upsert {"ID":"D46"}</t>
   </si>
 </sst>
 </file>
@@ -15875,12 +16255,12 @@
         <v>45</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>1478</v>
+        <v>1484</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>1481</v>
+        <v>1487</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>366</v>
@@ -15892,30 +16272,30 @@
         <v>49</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>1482</v>
+        <v>1488</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>1483</v>
+        <v>1489</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>1484</v>
+        <v>1490</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>1485</v>
+        <v>1491</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>686</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>1486</v>
+        <v>1492</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>1487</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>1488</v>
+        <v>1494</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>432</v>
@@ -15927,25 +16307,25 @@
         <v>49</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>1489</v>
+        <v>1495</v>
       </c>
       <c r="F3" s="6" t="s">
         <v>112</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>1490</v>
+        <v>1496</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>1491</v>
+        <v>1497</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>1492</v>
+        <v>1498</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>1493</v>
+        <v>1499</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>1494</v>
+        <v>1500</v>
       </c>
     </row>
   </sheetData>
@@ -41764,7 +42144,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -42654,6 +43034,32 @@
       </c>
       <c r="H36" s="6" t="s">
         <v>1289</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>1290</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>1291</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>1292</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>1293</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>1294</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>583</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>1129</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>1295</v>
       </c>
     </row>
   </sheetData>
@@ -42679,22 +43085,22 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>1290</v>
+        <v>1296</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1291</v>
+        <v>1297</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1292</v>
+        <v>1298</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1293</v>
+        <v>1299</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1294</v>
+        <v>1300</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>1067</v>
@@ -42702,1042 +43108,1042 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>1295</v>
+        <v>1301</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>1298</v>
+        <v>1304</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>1299</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>1300</v>
+        <v>1306</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>1302</v>
+        <v>1308</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>1303</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>1304</v>
+        <v>1310</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1305</v>
+        <v>1311</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>1306</v>
+        <v>1312</v>
       </c>
       <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>1307</v>
+        <v>1313</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1308</v>
+        <v>1314</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>1309</v>
+        <v>1315</v>
       </c>
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>1310</v>
+        <v>1316</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>1308</v>
+        <v>1314</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>1311</v>
+        <v>1317</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>1312</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>1313</v>
+        <v>1319</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>1314</v>
+        <v>1320</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>1315</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>1316</v>
+        <v>1322</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>1314</v>
+        <v>1320</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>1317</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>1318</v>
+        <v>1324</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>1319</v>
+        <v>1325</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>1320</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>1321</v>
+        <v>1327</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>1314</v>
+        <v>1320</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>1322</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>1323</v>
+        <v>1329</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>1314</v>
+        <v>1320</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>1324</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>1325</v>
+        <v>1331</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>118</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>1326</v>
+        <v>1332</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>1327</v>
+        <v>1333</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>1328</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>1329</v>
+        <v>1335</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>118</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>1326</v>
+        <v>1332</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>1330</v>
+        <v>1336</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>1331</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>1332</v>
+        <v>1338</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>132</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>1308</v>
+        <v>1314</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>1333</v>
+        <v>1339</v>
       </c>
       <c r="G14" s="2"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>1334</v>
+        <v>1340</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>132</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>1335</v>
+        <v>1341</v>
       </c>
       <c r="G15" s="2"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>1336</v>
+        <v>1342</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>132</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>1308</v>
+        <v>1314</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>1337</v>
+        <v>1343</v>
       </c>
       <c r="G16" s="2"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>1338</v>
+        <v>1344</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>132</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>1335</v>
+        <v>1341</v>
       </c>
       <c r="G17" s="2"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>1339</v>
+        <v>1345</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>132</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>1305</v>
+        <v>1311</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="G18" s="2"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>1341</v>
+        <v>1347</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>132</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>1335</v>
+        <v>1341</v>
       </c>
       <c r="G19" s="2"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>1342</v>
+        <v>1348</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>132</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>1343</v>
+        <v>1349</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>1335</v>
+        <v>1341</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>1344</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>1345</v>
+        <v>1351</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>132</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>1346</v>
+        <v>1352</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>1308</v>
+        <v>1314</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>1347</v>
+        <v>1353</v>
       </c>
       <c r="G21" s="2"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>1348</v>
+        <v>1354</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>132</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>1349</v>
+        <v>1355</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>1326</v>
+        <v>1332</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>1350</v>
+        <v>1356</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>1351</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>1352</v>
+        <v>1358</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>203</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>1308</v>
+        <v>1314</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>1353</v>
+        <v>1359</v>
       </c>
       <c r="G23" s="2"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>1354</v>
+        <v>1360</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>203</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>1355</v>
+        <v>1361</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>1356</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>1357</v>
+        <v>1363</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>203</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>1308</v>
+        <v>1314</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>1358</v>
+        <v>1364</v>
       </c>
       <c r="G25" s="2"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>1359</v>
+        <v>1365</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>203</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>1358</v>
+        <v>1364</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>1360</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>1361</v>
+        <v>1367</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>231</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>1305</v>
+        <v>1311</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>1362</v>
+        <v>1368</v>
       </c>
       <c r="G27" s="2"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>1363</v>
+        <v>1369</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>231</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>1364</v>
+        <v>1370</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>1305</v>
+        <v>1311</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>1365</v>
+        <v>1371</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>1366</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>1367</v>
+        <v>1373</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>231</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>1305</v>
+        <v>1311</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>1368</v>
+        <v>1374</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>1369</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>1370</v>
+        <v>1376</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>1371</v>
+        <v>1377</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>1372</v>
+        <v>1378</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>1373</v>
+        <v>1379</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>562</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>1374</v>
+        <v>1380</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>1375</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>1376</v>
+        <v>1382</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>1371</v>
+        <v>1377</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>1377</v>
+        <v>1383</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>1378</v>
+        <v>1384</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>556</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>1374</v>
+        <v>1380</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>1379</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>1380</v>
+        <v>1386</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>1371</v>
+        <v>1377</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>1381</v>
+        <v>1387</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>1378</v>
+        <v>1384</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>556</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>1374</v>
+        <v>1380</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>1382</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>1383</v>
+        <v>1389</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>1371</v>
+        <v>1377</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>1384</v>
+        <v>1390</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>1385</v>
+        <v>1391</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>556</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>1374</v>
+        <v>1380</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>1386</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>1387</v>
+        <v>1393</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>304</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>1388</v>
+        <v>1394</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>1389</v>
+        <v>1395</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>1390</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>1391</v>
+        <v>1397</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>304</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>1392</v>
+        <v>1398</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>1393</v>
+        <v>1399</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>1394</v>
+        <v>1400</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>1395</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>1396</v>
+        <v>1402</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>304</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>1308</v>
+        <v>1314</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>1397</v>
+        <v>1403</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>1398</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>1399</v>
+        <v>1405</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>304</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>1400</v>
+        <v>1406</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>1326</v>
+        <v>1332</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>1401</v>
+        <v>1407</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>1402</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>1403</v>
+        <v>1409</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>328</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>1326</v>
+        <v>1332</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>1404</v>
+        <v>1410</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>1405</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>1406</v>
+        <v>1412</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>328</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>1407</v>
+        <v>1413</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>1308</v>
+        <v>1314</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>1408</v>
+        <v>1414</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>1409</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>1410</v>
+        <v>1416</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>328</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>1411</v>
+        <v>1417</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>1308</v>
+        <v>1314</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>1412</v>
+        <v>1418</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>1413</v>
+        <v>1419</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>1414</v>
+        <v>1420</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>328</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>1415</v>
+        <v>1421</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>1416</v>
+        <v>1422</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>1417</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>1418</v>
+        <v>1424</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>353</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>1388</v>
+        <v>1394</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>1419</v>
+        <v>1425</v>
       </c>
       <c r="G42" s="2"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>1420</v>
+        <v>1426</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>353</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>1421</v>
+        <v>1427</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>1422</v>
+        <v>1428</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>1423</v>
+        <v>1429</v>
       </c>
       <c r="G43" s="2"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>1424</v>
+        <v>1430</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>353</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>1425</v>
+        <v>1431</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>1422</v>
+        <v>1428</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>1423</v>
+        <v>1429</v>
       </c>
       <c r="G44" s="2"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>1426</v>
+        <v>1432</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>353</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>1427</v>
+        <v>1433</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>1422</v>
+        <v>1428</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>1423</v>
+        <v>1429</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>1428</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>1429</v>
+        <v>1435</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>353</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>1430</v>
+        <v>1436</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>1308</v>
+        <v>1314</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>1397</v>
+        <v>1403</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>1431</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>1432</v>
+        <v>1438</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>380</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>1388</v>
+        <v>1394</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>1433</v>
+        <v>1439</v>
       </c>
       <c r="G47" s="2"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>1434</v>
+        <v>1440</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>380</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>1411</v>
+        <v>1417</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>1393</v>
+        <v>1399</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>628</v>
@@ -43746,342 +44152,342 @@
         <v>118</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>1435</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>1436</v>
+        <v>1442</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>380</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>1437</v>
+        <v>1443</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>1308</v>
+        <v>1314</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>1438</v>
+        <v>1444</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>1439</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>1440</v>
+        <v>1446</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>380</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>1441</v>
+        <v>1447</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>1422</v>
+        <v>1428</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>1423</v>
+        <v>1429</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>1442</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>1443</v>
+        <v>1449</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>399</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>1308</v>
+        <v>1314</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>1444</v>
+        <v>1450</v>
       </c>
       <c r="G51" s="2"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>1445</v>
+        <v>1451</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>399</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>1444</v>
+        <v>1450</v>
       </c>
       <c r="G52" s="2"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>1446</v>
+        <v>1452</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>445</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>1447</v>
+        <v>1453</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>1326</v>
+        <v>1332</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>1448</v>
+        <v>1454</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>1449</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>1450</v>
+        <v>1456</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>445</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>1326</v>
+        <v>1332</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>1451</v>
+        <v>1457</v>
       </c>
       <c r="G54" s="2"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>1452</v>
+        <v>1458</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>445</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>1453</v>
+        <v>1459</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>1454</v>
+        <v>1460</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>1455</v>
+        <v>1461</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>418</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>1456</v>
+        <v>1462</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>1457</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>1458</v>
+        <v>1464</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>1459</v>
+        <v>1465</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>1305</v>
+        <v>1311</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>1460</v>
+        <v>1466</v>
       </c>
       <c r="G57" s="2"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>1461</v>
+        <v>1467</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>1459</v>
+        <v>1465</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>1308</v>
+        <v>1314</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>1462</v>
+        <v>1468</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>1463</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>1464</v>
+        <v>1470</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>1459</v>
+        <v>1465</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>1305</v>
+        <v>1311</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>628</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>1465</v>
+        <v>1471</v>
       </c>
       <c r="G59" s="2"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>1466</v>
+        <v>1472</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>1459</v>
+        <v>1465</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>1467</v>
+        <v>1473</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>1305</v>
+        <v>1311</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>1468</v>
+        <v>1474</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>1469</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>1470</v>
+        <v>1476</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>108</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>1296</v>
+        <v>1302</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>1305</v>
+        <v>1311</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>1471</v>
+        <v>1477</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>1472</v>
+        <v>1478</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>1473</v>
+        <v>1479</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>108</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>1437</v>
+        <v>1443</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>1305</v>
+        <v>1311</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>1474</v>
+        <v>1480</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>1475</v>
+        <v>1481</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>1476</v>
+        <v>1482</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>432</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>1301</v>
+        <v>1307</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>1297</v>
+        <v>1303</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>868</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>1302</v>
+        <v>1308</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>1477</v>
+        <v>1483</v>
       </c>
     </row>
   </sheetData>
@@ -44093,7 +44499,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -44106,922 +44512,1002 @@
   <sheetData>
     <row r="1" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>1495</v>
+        <v>1501</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>1496</v>
+        <v>1502</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>1497</v>
+        <v>1503</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>1498</v>
+        <v>1504</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>1499</v>
+        <v>1505</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>1500</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>1501</v>
+        <v>1507</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>1502</v>
+        <v>1508</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>1503</v>
+        <v>1509</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>1504</v>
+        <v>1510</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>1505</v>
+        <v>1511</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>1506</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>1507</v>
+        <v>1513</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>1502</v>
+        <v>1508</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>1508</v>
+        <v>1514</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>1509</v>
+        <v>1515</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>1510</v>
+        <v>1516</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>1511</v>
+        <v>1517</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>1512</v>
+        <v>1518</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>1502</v>
+        <v>1508</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>1503</v>
+        <v>1509</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>1513</v>
+        <v>1519</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>1514</v>
+        <v>1520</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>1515</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>1516</v>
+        <v>1522</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>1502</v>
+        <v>1508</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>1517</v>
+        <v>1523</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>1518</v>
+        <v>1524</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>1519</v>
+        <v>1525</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>1520</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>1521</v>
+        <v>1527</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>1502</v>
+        <v>1508</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>1522</v>
+        <v>1528</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>1523</v>
+        <v>1529</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>1524</v>
+        <v>1530</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>1526</v>
+        <v>1532</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>1502</v>
+        <v>1508</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>1527</v>
+        <v>1533</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>1528</v>
+        <v>1534</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>1529</v>
+        <v>1535</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>1479</v>
+        <v>1485</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>1502</v>
+        <v>1508</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>1503</v>
+        <v>1509</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>1530</v>
+        <v>1536</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>1531</v>
+        <v>1537</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>1532</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>1533</v>
+        <v>1539</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>1534</v>
+        <v>1540</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>1535</v>
+        <v>1541</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>1536</v>
+        <v>1542</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>1537</v>
+        <v>1543</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>1538</v>
+        <v>1544</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>1534</v>
+        <v>1540</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>1539</v>
+        <v>1545</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>1540</v>
+        <v>1546</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>1541</v>
+        <v>1547</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>1542</v>
+        <v>1548</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>1543</v>
+        <v>1549</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>1544</v>
+        <v>1550</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>1545</v>
+        <v>1551</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>1546</v>
+        <v>1552</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>1547</v>
+        <v>1553</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>1548</v>
+        <v>1554</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>1543</v>
+        <v>1549</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>1549</v>
+        <v>1555</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>1550</v>
+        <v>1556</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>1551</v>
+        <v>1557</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>1552</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>1553</v>
+        <v>1559</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>1554</v>
+        <v>1560</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>1555</v>
+        <v>1561</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>1556</v>
+        <v>1562</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>1557</v>
+        <v>1563</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>1558</v>
+        <v>1564</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>1559</v>
+        <v>1565</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>1560</v>
+        <v>1566</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>1539</v>
+        <v>1545</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>1561</v>
+        <v>1567</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>1562</v>
+        <v>1568</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>1563</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>1564</v>
+        <v>1570</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>1560</v>
+        <v>1566</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>1565</v>
+        <v>1571</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>1566</v>
+        <v>1572</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>1567</v>
+        <v>1573</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>1568</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>1569</v>
+        <v>1575</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>1560</v>
+        <v>1566</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>1570</v>
+        <v>1576</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>1571</v>
+        <v>1577</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>1572</v>
+        <v>1578</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>1573</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>1574</v>
+        <v>1580</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>1560</v>
+        <v>1566</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>1575</v>
+        <v>1581</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>1576</v>
+        <v>1582</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>1577</v>
+        <v>1583</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>1578</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>1579</v>
+        <v>1585</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>1560</v>
+        <v>1566</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>1580</v>
+        <v>1586</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>1581</v>
+        <v>1587</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>1582</v>
+        <v>1588</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>1583</v>
+        <v>1589</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>1584</v>
+        <v>1590</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>1585</v>
+        <v>1591</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>1586</v>
+        <v>1592</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>1587</v>
+        <v>1593</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>1588</v>
+        <v>1594</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>1589</v>
+        <v>1595</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>1590</v>
+        <v>1596</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>1585</v>
+        <v>1591</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>1591</v>
+        <v>1597</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>1592</v>
+        <v>1598</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>1593</v>
+        <v>1599</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>1594</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>1595</v>
+        <v>1601</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>1596</v>
+        <v>1602</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>1597</v>
+        <v>1603</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>1598</v>
+        <v>1604</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>1599</v>
+        <v>1605</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>1600</v>
+        <v>1606</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>1596</v>
+        <v>1602</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>1601</v>
+        <v>1607</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>1602</v>
+        <v>1608</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>1603</v>
+        <v>1609</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>1604</v>
+        <v>1610</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>1596</v>
+        <v>1602</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>1605</v>
+        <v>1611</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>1606</v>
+        <v>1612</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>1608</v>
+        <v>1614</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>1596</v>
+        <v>1602</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>1609</v>
+        <v>1615</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>1610</v>
+        <v>1616</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>1611</v>
+        <v>1617</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>1612</v>
+        <v>1618</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>1613</v>
+        <v>1619</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>1596</v>
+        <v>1602</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>1614</v>
+        <v>1620</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>1615</v>
+        <v>1621</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>1616</v>
+        <v>1622</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>1617</v>
+        <v>1623</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>1596</v>
+        <v>1602</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>1618</v>
+        <v>1624</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>1619</v>
+        <v>1625</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>1620</v>
+        <v>1626</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>1621</v>
+        <v>1627</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>1596</v>
+        <v>1602</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>1622</v>
+        <v>1628</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>1623</v>
+        <v>1629</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>1624</v>
+        <v>1630</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>1625</v>
+        <v>1631</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>1596</v>
+        <v>1602</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>1626</v>
+        <v>1632</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>1627</v>
+        <v>1633</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>1628</v>
+        <v>1634</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>1629</v>
+        <v>1635</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>1630</v>
+        <v>1636</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>1596</v>
+        <v>1602</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>1631</v>
+        <v>1637</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>1632</v>
+        <v>1638</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>1633</v>
+        <v>1639</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>1634</v>
+        <v>1640</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>1596</v>
+        <v>1602</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>1635</v>
+        <v>1641</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>1636</v>
+        <v>1642</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>1637</v>
+        <v>1643</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>1638</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>1639</v>
+        <v>1645</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>1596</v>
+        <v>1602</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>1640</v>
+        <v>1646</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>1641</v>
+        <v>1647</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>1642</v>
+        <v>1648</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>1643</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>1644</v>
+        <v>1650</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>1645</v>
+        <v>1651</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>1646</v>
+        <v>1652</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>1647</v>
+        <v>1653</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>1648</v>
+        <v>1654</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>1649</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>1650</v>
+        <v>1656</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>1596</v>
+        <v>1602</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>1651</v>
+        <v>1657</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>1652</v>
+        <v>1658</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>1653</v>
+        <v>1659</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>1654</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>1655</v>
+        <v>1661</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>1645</v>
+        <v>1651</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>1656</v>
+        <v>1662</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>1657</v>
+        <v>1663</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>1658</v>
+        <v>1664</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>1659</v>
+        <v>1665</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>1660</v>
+        <v>1666</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>1645</v>
+        <v>1651</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>1661</v>
+        <v>1667</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>1662</v>
+        <v>1668</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>1663</v>
+        <v>1669</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>1664</v>
+        <v>1670</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>1645</v>
+        <v>1651</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>1665</v>
+        <v>1671</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>1666</v>
+        <v>1672</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>1667</v>
+        <v>1673</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>1668</v>
+        <v>1674</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>1669</v>
+        <v>1675</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>1670</v>
+        <v>1676</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>1671</v>
+        <v>1677</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>1672</v>
+        <v>1678</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
-        <v>1673</v>
+        <v>1679</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>1669</v>
+        <v>1675</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>1674</v>
+        <v>1680</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>1675</v>
+        <v>1681</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>1676</v>
+        <v>1682</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>1677</v>
+        <v>1683</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>1480</v>
+        <v>1486</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>1669</v>
+        <v>1675</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>1678</v>
+        <v>1684</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>1679</v>
+        <v>1685</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>1680</v>
+        <v>1686</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>1681</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>1682</v>
+        <v>1688</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>1669</v>
+        <v>1675</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>1683</v>
+        <v>1689</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>1684</v>
+        <v>1690</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>1685</v>
+        <v>1691</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>1686</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>1487</v>
+        <v>1493</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>1687</v>
+        <v>1693</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>1688</v>
+        <v>1694</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>1689</v>
+        <v>1695</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>1690</v>
+        <v>1696</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>1691</v>
+        <v>1697</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
-        <v>1494</v>
+        <v>1500</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>1687</v>
+        <v>1693</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>1692</v>
+        <v>1698</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>1693</v>
+        <v>1699</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>1694</v>
+        <v>1700</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>1695</v>
+        <v>1701</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
-        <v>1696</v>
+        <v>1702</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>1687</v>
+        <v>1693</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>1697</v>
+        <v>1703</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>1698</v>
+        <v>1704</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>1699</v>
+        <v>1705</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>1700</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
-        <v>1701</v>
+        <v>1707</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>1687</v>
+        <v>1693</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>1702</v>
+        <v>1708</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>1703</v>
+        <v>1709</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>1704</v>
+        <v>1710</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>1525</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>1705</v>
+        <v>1711</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>1687</v>
+        <v>1693</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>1706</v>
+        <v>1712</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>1707</v>
+        <v>1713</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>1708</v>
+        <v>1714</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>1709</v>
+        <v>1715</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>1710</v>
+        <v>1716</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>1687</v>
+        <v>1693</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>1711</v>
+        <v>1717</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>1712</v>
+        <v>1718</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>1713</v>
+        <v>1719</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>1714</v>
+        <v>1720</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
+        <v>1721</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>1693</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>1722</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>1723</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>1724</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>1531</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="6" t="s">
+        <v>1725</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>1693</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>1726</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>1727</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>1728</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>1531</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="6" t="s">
+        <v>1729</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>1730</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>1731</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>1732</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>1733</v>
+      </c>
+      <c r="F49" s="6" t="s">
+        <v>1531</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="6" t="s">
+        <v>1734</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>1730</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>1735</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>1736</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>1737</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>1738</v>
       </c>
     </row>
   </sheetData>
@@ -45077,7 +45563,7 @@
         <v>553</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>1478</v>
+        <v>1484</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -45109,7 +45595,7 @@
         <v>819</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>1479</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -45141,7 +45627,7 @@
         <v>819</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>1479</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -45173,7 +45659,7 @@
         <v>819</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>1479</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -45205,7 +45691,7 @@
         <v>819</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>1479</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -45237,7 +45723,7 @@
         <v>819</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>1479</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -45269,7 +45755,7 @@
         <v>819</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>1479</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -45301,7 +45787,7 @@
         <v>819</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>1479</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -45333,7 +45819,7 @@
         <v>819</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>1479</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -45365,7 +45851,7 @@
         <v>819</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>1479</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -45397,7 +45883,7 @@
         <v>819</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>1479</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -45429,7 +45915,7 @@
         <v>819</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>1480</v>
+        <v>1486</v>
       </c>
     </row>
   </sheetData>

</xml_diff>